<commit_message>
v1.04 Sanitize Species upstream and remove redundant plotting code
Moved species sanitization to the import stage, removed the redundant sanitization block from the plotting script, and added the same upstream sanitization to Jon's elecfish workflow.
</commit_message>
<xml_diff>
--- a/01_data/01_raw_files/Fixed_fish_widths_DraftExcelAnalysis_Feb2026.xlsx
+++ b/01_data/01_raw_files/Fixed_fish_widths_DraftExcelAnalysis_Feb2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RIZZUTOM\Desktop\GitHub Projects\2026_Reddick_fish_morphology\01_data\01_raw_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA0F3796-C651-472A-B1D0-605469A47CFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D8C15C2-8299-4F88-A70E-1C5083081186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,11 +17,11 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$486</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$486</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -7174,7 +7174,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C6EF6C66-FE5E-494C-94DC-2E9CD6A79F69}" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C6EF6C66-FE5E-494C-94DC-2E9CD6A79F69}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="L2:L24" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -13868,31 +13868,31 @@
       <c r="J205" s="6"/>
     </row>
     <row r="206" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A206" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B206" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C206" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="D206" s="11">
+      <c r="A206" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B206" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C206" t="s">
+        <v>125</v>
+      </c>
+      <c r="D206" s="10">
         <v>45944</v>
       </c>
-      <c r="E206" s="2" t="s">
+      <c r="E206" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F206" s="2">
-        <v>438</v>
-      </c>
-      <c r="G206" s="2">
-        <v>650</v>
-      </c>
-      <c r="H206" s="2">
-        <v>1670</v>
-      </c>
-      <c r="I206" s="2" t="s">
+      <c r="F206" s="6">
+        <v>344</v>
+      </c>
+      <c r="G206" s="6">
+        <v>55</v>
+      </c>
+      <c r="H206" s="6">
+        <v>900</v>
+      </c>
+      <c r="I206" s="6" t="s">
         <v>88</v>
       </c>
     </row>
@@ -13901,7 +13901,7 @@
         <v>11</v>
       </c>
       <c r="B207" s="6" t="s">
-        <v>61</v>
+        <v>93</v>
       </c>
       <c r="C207" t="s">
         <v>125</v>
@@ -13913,13 +13913,13 @@
         <v>21</v>
       </c>
       <c r="F207" s="6">
-        <v>470</v>
+        <v>86</v>
       </c>
       <c r="G207" s="6">
-        <v>90</v>
+        <v>8</v>
       </c>
       <c r="H207" s="6">
-        <v>2480</v>
+        <v>10</v>
       </c>
       <c r="I207" s="6" t="s">
         <v>88</v>
@@ -13927,29 +13927,32 @@
       <c r="J207" s="6"/>
     </row>
     <row r="208" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A208" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B208" s="2" t="s">
-        <v>77</v>
+      <c r="A208" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B208" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="C208" t="s">
         <v>125</v>
       </c>
-      <c r="D208" s="11">
-        <v>45791</v>
-      </c>
-      <c r="E208" s="2" t="s">
+      <c r="D208" s="10">
+        <v>45944</v>
+      </c>
+      <c r="E208" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F208" s="2">
-        <v>470</v>
-      </c>
-      <c r="G208" s="2">
-        <v>86</v>
-      </c>
-      <c r="H208" s="2">
-        <v>2460</v>
+      <c r="F208" s="6">
+        <v>92</v>
+      </c>
+      <c r="G208" s="6">
+        <v>10</v>
+      </c>
+      <c r="H208" s="6">
+        <v>10</v>
+      </c>
+      <c r="I208" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="J208" s="6"/>
     </row>
@@ -13958,25 +13961,25 @@
         <v>11</v>
       </c>
       <c r="B209" s="6" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="C209" t="s">
         <v>125</v>
       </c>
       <c r="D209" s="10">
-        <v>45791</v>
+        <v>45944</v>
       </c>
       <c r="E209" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F209" s="6">
-        <v>470</v>
+        <v>92</v>
       </c>
       <c r="G209" s="6">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="H209" s="6">
-        <v>2460</v>
+        <v>12</v>
       </c>
       <c r="I209" s="6" t="s">
         <v>88</v>
@@ -13984,29 +13987,32 @@
       <c r="J209" s="6"/>
     </row>
     <row r="210" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A210" t="s">
-        <v>11</v>
-      </c>
-      <c r="B210" t="s">
-        <v>51</v>
+      <c r="A210" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B210" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="C210" t="s">
         <v>125</v>
       </c>
-      <c r="D210" s="1">
-        <v>45791</v>
-      </c>
-      <c r="E210" t="s">
+      <c r="D210" s="10">
+        <v>45944</v>
+      </c>
+      <c r="E210" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F210">
-        <v>380</v>
-      </c>
-      <c r="G210">
-        <v>80</v>
-      </c>
-      <c r="H210">
-        <v>1450</v>
+      <c r="F210" s="6">
+        <v>95</v>
+      </c>
+      <c r="G210" s="6">
+        <v>10</v>
+      </c>
+      <c r="H210" s="6">
+        <v>10</v>
+      </c>
+      <c r="I210" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="J210" s="6"/>
     </row>
@@ -14015,25 +14021,25 @@
         <v>11</v>
       </c>
       <c r="B211" s="6" t="s">
-        <v>51</v>
+        <v>93</v>
       </c>
       <c r="C211" t="s">
         <v>125</v>
       </c>
       <c r="D211" s="10">
-        <v>45791</v>
+        <v>45944</v>
       </c>
       <c r="E211" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F211" s="6">
-        <v>380</v>
+        <v>96</v>
       </c>
       <c r="G211" s="6">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="H211" s="6">
-        <v>1450</v>
+        <v>13</v>
       </c>
       <c r="I211" s="6" t="s">
         <v>88</v>
@@ -14041,32 +14047,32 @@
       <c r="J211" s="6"/>
     </row>
     <row r="212" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A212" t="s">
-        <v>11</v>
-      </c>
-      <c r="B212" t="s">
-        <v>77</v>
+      <c r="A212" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B212" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="C212" t="s">
         <v>125</v>
       </c>
-      <c r="D212" s="1">
-        <v>45803</v>
-      </c>
-      <c r="E212" t="s">
+      <c r="D212" s="10">
+        <v>45944</v>
+      </c>
+      <c r="E212" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F212">
-        <v>463</v>
-      </c>
-      <c r="G212">
-        <v>80</v>
-      </c>
-      <c r="H212">
-        <v>2140</v>
-      </c>
-      <c r="I212" t="s">
-        <v>78</v>
+      <c r="F212" s="6">
+        <v>99</v>
+      </c>
+      <c r="G212" s="6">
+        <v>10</v>
+      </c>
+      <c r="H212" s="6">
+        <v>13</v>
+      </c>
+      <c r="I212" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="J212" s="6"/>
     </row>
@@ -14075,25 +14081,25 @@
         <v>11</v>
       </c>
       <c r="B213" s="6" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="C213" t="s">
         <v>125</v>
       </c>
       <c r="D213" s="10">
-        <v>45803</v>
+        <v>45944</v>
       </c>
       <c r="E213" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F213" s="6">
-        <v>463</v>
+        <v>100</v>
       </c>
       <c r="G213" s="6">
-        <v>80</v>
+        <v>13</v>
       </c>
       <c r="H213" s="6">
-        <v>2140</v>
+        <v>15</v>
       </c>
       <c r="I213" s="6" t="s">
         <v>88</v>
@@ -14105,25 +14111,25 @@
         <v>11</v>
       </c>
       <c r="B214" s="6" t="s">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="C214" t="s">
         <v>125</v>
       </c>
       <c r="D214" s="10">
-        <v>45951</v>
+        <v>45945</v>
       </c>
       <c r="E214" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F214" s="6">
-        <v>494</v>
+        <v>102</v>
       </c>
       <c r="G214" s="6">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="H214" s="6">
-        <v>2390</v>
+        <v>16</v>
       </c>
       <c r="I214" s="6" t="s">
         <v>88</v>
@@ -14135,25 +14141,25 @@
         <v>11</v>
       </c>
       <c r="B215" s="6" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="C215" t="s">
         <v>125</v>
       </c>
       <c r="D215" s="10">
-        <v>45946</v>
+        <v>45945</v>
       </c>
       <c r="E215" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F215" s="6">
-        <v>465</v>
+        <v>106</v>
       </c>
       <c r="G215" s="6">
-        <v>80</v>
+        <v>18</v>
       </c>
       <c r="H215" s="6">
-        <v>2430</v>
+        <v>10</v>
       </c>
       <c r="I215" s="6" t="s">
         <v>88</v>
@@ -14161,29 +14167,32 @@
       <c r="J215" s="6"/>
     </row>
     <row r="216" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A216" t="s">
-        <v>11</v>
-      </c>
-      <c r="B216" t="s">
-        <v>45</v>
+      <c r="A216" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B216" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="C216" t="s">
         <v>125</v>
       </c>
-      <c r="D216" s="1">
-        <v>45791</v>
-      </c>
-      <c r="E216" t="s">
+      <c r="D216" s="10">
+        <v>45944</v>
+      </c>
+      <c r="E216" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F216">
-        <v>424</v>
-      </c>
-      <c r="G216">
-        <v>76</v>
-      </c>
-      <c r="H216">
-        <v>1610</v>
+      <c r="F216" s="6">
+        <v>106</v>
+      </c>
+      <c r="G216" s="6">
+        <v>15</v>
+      </c>
+      <c r="H216" s="6">
+        <v>25</v>
+      </c>
+      <c r="I216" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="J216" s="6"/>
     </row>
@@ -14192,25 +14201,25 @@
         <v>11</v>
       </c>
       <c r="B217" s="6" t="s">
-        <v>45</v>
+        <v>93</v>
       </c>
       <c r="C217" t="s">
         <v>125</v>
       </c>
       <c r="D217" s="10">
-        <v>45791</v>
+        <v>45944</v>
       </c>
       <c r="E217" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F217" s="6">
-        <v>424</v>
+        <v>107</v>
       </c>
       <c r="G217" s="6">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="H217" s="6">
-        <v>1610</v>
+        <v>27</v>
       </c>
       <c r="I217" s="6" t="s">
         <v>88</v>
@@ -14218,29 +14227,32 @@
       <c r="J217" s="6"/>
     </row>
     <row r="218" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A218" t="s">
-        <v>11</v>
-      </c>
-      <c r="B218" t="s">
-        <v>45</v>
+      <c r="A218" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B218" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="C218" t="s">
         <v>125</v>
       </c>
-      <c r="D218" s="1">
-        <v>45791</v>
-      </c>
-      <c r="E218" t="s">
+      <c r="D218" s="10">
+        <v>45944</v>
+      </c>
+      <c r="E218" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F218">
-        <v>405</v>
-      </c>
-      <c r="G218">
-        <v>76</v>
-      </c>
-      <c r="H218">
-        <v>1620</v>
+      <c r="F218" s="6">
+        <v>107</v>
+      </c>
+      <c r="G218" s="6">
+        <v>12</v>
+      </c>
+      <c r="H218" s="6">
+        <v>17</v>
+      </c>
+      <c r="I218" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="J218" s="6"/>
     </row>
@@ -14249,25 +14261,25 @@
         <v>11</v>
       </c>
       <c r="B219" s="6" t="s">
-        <v>45</v>
+        <v>93</v>
       </c>
       <c r="C219" t="s">
         <v>125</v>
       </c>
       <c r="D219" s="10">
-        <v>45791</v>
+        <v>45945</v>
       </c>
       <c r="E219" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F219" s="6">
-        <v>405</v>
+        <v>112</v>
       </c>
       <c r="G219" s="6">
-        <v>76</v>
+        <v>10</v>
       </c>
       <c r="H219" s="6">
-        <v>1620</v>
+        <v>21</v>
       </c>
       <c r="I219" s="6" t="s">
         <v>88</v>
@@ -14275,29 +14287,32 @@
       <c r="J219" s="6"/>
     </row>
     <row r="220" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A220" t="s">
-        <v>11</v>
-      </c>
-      <c r="B220" t="s">
-        <v>51</v>
+      <c r="A220" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B220" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="C220" t="s">
         <v>125</v>
       </c>
-      <c r="D220" s="1">
-        <v>45791</v>
-      </c>
-      <c r="E220" t="s">
+      <c r="D220" s="10">
+        <v>45945</v>
+      </c>
+      <c r="E220" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F220">
-        <v>426</v>
-      </c>
-      <c r="G220">
-        <v>74</v>
-      </c>
-      <c r="H220">
-        <v>1700</v>
+      <c r="F220" s="6">
+        <v>123</v>
+      </c>
+      <c r="G220" s="6">
+        <v>10</v>
+      </c>
+      <c r="H220" s="6">
+        <v>25</v>
+      </c>
+      <c r="I220" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="J220" s="6"/>
     </row>
@@ -14306,25 +14321,25 @@
         <v>11</v>
       </c>
       <c r="B221" s="6" t="s">
-        <v>51</v>
+        <v>93</v>
       </c>
       <c r="C221" t="s">
         <v>125</v>
       </c>
       <c r="D221" s="10">
-        <v>45791</v>
+        <v>45944</v>
       </c>
       <c r="E221" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F221" s="6">
-        <v>426</v>
+        <v>126</v>
       </c>
       <c r="G221" s="6">
-        <v>74</v>
+        <v>10</v>
       </c>
       <c r="H221" s="6">
-        <v>1700</v>
+        <v>28</v>
       </c>
       <c r="I221" s="6" t="s">
         <v>88</v>
@@ -14332,29 +14347,32 @@
       <c r="J221" s="6"/>
     </row>
     <row r="222" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A222" t="s">
-        <v>11</v>
-      </c>
-      <c r="B222" t="s">
-        <v>12</v>
+      <c r="A222" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B222" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="C222" t="s">
         <v>125</v>
       </c>
-      <c r="D222" s="1">
-        <v>45803</v>
-      </c>
-      <c r="E222" t="s">
+      <c r="D222" s="10">
+        <v>45944</v>
+      </c>
+      <c r="E222" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F222">
-        <v>414</v>
-      </c>
-      <c r="G222">
-        <v>70</v>
-      </c>
-      <c r="H222">
-        <v>1640</v>
+      <c r="F222" s="6">
+        <v>130</v>
+      </c>
+      <c r="G222" s="6">
+        <v>15</v>
+      </c>
+      <c r="H222" s="6">
+        <v>34</v>
+      </c>
+      <c r="I222" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="J222" s="6"/>
     </row>
@@ -14363,25 +14381,25 @@
         <v>11</v>
       </c>
       <c r="B223" s="6" t="s">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="C223" t="s">
         <v>125</v>
       </c>
       <c r="D223" s="10">
-        <v>45803</v>
+        <v>45944</v>
       </c>
       <c r="E223" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F223" s="6">
-        <v>414</v>
+        <v>130</v>
       </c>
       <c r="G223" s="6">
-        <v>70</v>
+        <v>12</v>
       </c>
       <c r="H223" s="6">
-        <v>1640</v>
+        <v>34</v>
       </c>
       <c r="I223" s="6" t="s">
         <v>88</v>
@@ -14399,19 +14417,19 @@
         <v>125</v>
       </c>
       <c r="D224" s="1">
-        <v>45799</v>
+        <v>45803</v>
       </c>
       <c r="E224" t="s">
         <v>21</v>
       </c>
       <c r="F224">
-        <v>435</v>
+        <v>145</v>
       </c>
       <c r="G224">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="H224">
-        <v>1810</v>
+        <v>40</v>
       </c>
       <c r="J224" s="6"/>
     </row>
@@ -14426,19 +14444,19 @@
         <v>125</v>
       </c>
       <c r="D225" s="10">
-        <v>45799</v>
+        <v>45803</v>
       </c>
       <c r="E225" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F225" s="6">
-        <v>435</v>
+        <v>145</v>
       </c>
       <c r="G225" s="6">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="H225" s="6">
-        <v>1810</v>
+        <v>40</v>
       </c>
       <c r="I225" s="6" t="s">
         <v>88</v>
@@ -14446,29 +14464,32 @@
       <c r="J225" s="6"/>
     </row>
     <row r="226" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A226" t="s">
-        <v>11</v>
-      </c>
-      <c r="B226" t="s">
-        <v>55</v>
+      <c r="A226" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B226" s="6" t="s">
+        <v>92</v>
       </c>
       <c r="C226" t="s">
         <v>125</v>
       </c>
-      <c r="D226" s="1">
-        <v>45799</v>
-      </c>
-      <c r="E226" t="s">
+      <c r="D226" s="10">
+        <v>45944</v>
+      </c>
+      <c r="E226" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F226">
-        <v>450</v>
-      </c>
-      <c r="G226">
-        <v>70</v>
-      </c>
-      <c r="H226">
-        <v>2000</v>
+      <c r="F226" s="6">
+        <v>148</v>
+      </c>
+      <c r="G226" s="6">
+        <v>15</v>
+      </c>
+      <c r="H226" s="6">
+        <v>52</v>
+      </c>
+      <c r="I226" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="J226" s="6"/>
     </row>
@@ -14477,25 +14498,25 @@
         <v>11</v>
       </c>
       <c r="B227" s="6" t="s">
-        <v>55</v>
+        <v>92</v>
       </c>
       <c r="C227" t="s">
         <v>125</v>
       </c>
       <c r="D227" s="10">
-        <v>45799</v>
+        <v>45945</v>
       </c>
       <c r="E227" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F227" s="6">
-        <v>450</v>
+        <v>149</v>
       </c>
       <c r="G227" s="6">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="H227" s="6">
-        <v>2000</v>
+        <v>50</v>
       </c>
       <c r="I227" s="6" t="s">
         <v>88</v>
@@ -14503,88 +14524,91 @@
       <c r="J227" s="6"/>
     </row>
     <row r="228" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A228" t="s">
-        <v>11</v>
-      </c>
-      <c r="B228" t="s">
-        <v>73</v>
+      <c r="A228" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B228" s="6" t="s">
+        <v>79</v>
       </c>
       <c r="C228" t="s">
         <v>125</v>
       </c>
-      <c r="D228" s="1">
-        <v>45791</v>
-      </c>
-      <c r="E228" t="s">
+      <c r="D228" s="10">
+        <v>45799</v>
+      </c>
+      <c r="E228" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F228">
-        <v>408</v>
-      </c>
-      <c r="G228">
-        <v>68</v>
-      </c>
-      <c r="H228">
-        <v>1470</v>
-      </c>
-      <c r="I228" t="s">
-        <v>74</v>
+      <c r="F228" s="6">
+        <v>155</v>
+      </c>
+      <c r="G228" s="6">
+        <v>41</v>
+      </c>
+      <c r="H228" s="6">
+        <v>150</v>
+      </c>
+      <c r="I228" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="J228" s="6"/>
     </row>
     <row r="229" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A229" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B229" s="6" t="s">
-        <v>73</v>
+      <c r="A229" t="s">
+        <v>11</v>
+      </c>
+      <c r="B229" t="s">
+        <v>79</v>
       </c>
       <c r="C229" t="s">
         <v>125</v>
       </c>
-      <c r="D229" s="10">
-        <v>45791</v>
-      </c>
-      <c r="E229" s="6" t="s">
+      <c r="D229" s="1">
+        <v>45799</v>
+      </c>
+      <c r="E229" t="s">
         <v>21</v>
       </c>
-      <c r="F229" s="6">
-        <v>408</v>
-      </c>
-      <c r="G229" s="6">
-        <v>68</v>
-      </c>
-      <c r="H229" s="6">
-        <v>1470</v>
-      </c>
-      <c r="I229" s="6" t="s">
-        <v>88</v>
+      <c r="F229">
+        <v>155</v>
+      </c>
+      <c r="G229" s="2">
+        <v>15</v>
+      </c>
+      <c r="H229">
+        <v>41</v>
+      </c>
+      <c r="I229" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="230" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A230" t="s">
-        <v>11</v>
-      </c>
-      <c r="B230" t="s">
-        <v>55</v>
+      <c r="A230" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B230" s="6" t="s">
+        <v>93</v>
       </c>
       <c r="C230" t="s">
         <v>125</v>
       </c>
-      <c r="D230" s="1">
-        <v>45791</v>
-      </c>
-      <c r="E230" t="s">
+      <c r="D230" s="10">
+        <v>45944</v>
+      </c>
+      <c r="E230" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F230">
-        <v>458</v>
-      </c>
-      <c r="G230">
-        <v>68</v>
-      </c>
-      <c r="H230">
-        <v>1680</v>
+      <c r="F230" s="6">
+        <v>156</v>
+      </c>
+      <c r="G230" s="6">
+        <v>20</v>
+      </c>
+      <c r="H230" s="6">
+        <v>62</v>
+      </c>
+      <c r="I230" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="J230" s="6"/>
     </row>
@@ -14593,25 +14617,25 @@
         <v>11</v>
       </c>
       <c r="B231" s="6" t="s">
-        <v>55</v>
+        <v>92</v>
       </c>
       <c r="C231" t="s">
         <v>125</v>
       </c>
       <c r="D231" s="10">
-        <v>45791</v>
+        <v>45944</v>
       </c>
       <c r="E231" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F231" s="6">
-        <v>458</v>
+        <v>156</v>
       </c>
       <c r="G231" s="6">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="H231" s="6">
-        <v>1680</v>
+        <v>57</v>
       </c>
       <c r="I231" s="6" t="s">
         <v>88</v>
@@ -14634,13 +14658,13 @@
         <v>21</v>
       </c>
       <c r="F232" s="6">
-        <v>340</v>
+        <v>184</v>
       </c>
       <c r="G232" s="6">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="H232" s="6">
-        <v>1250</v>
+        <v>94</v>
       </c>
       <c r="I232" s="6" t="s">
         <v>88</v>
@@ -14652,25 +14676,25 @@
         <v>11</v>
       </c>
       <c r="B233" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="C233" t="s">
         <v>125</v>
       </c>
       <c r="D233" s="1">
-        <v>45799</v>
+        <v>45792</v>
       </c>
       <c r="E233" t="s">
         <v>21</v>
       </c>
       <c r="F233">
-        <v>417</v>
-      </c>
-      <c r="G233">
-        <v>65</v>
-      </c>
-      <c r="H233">
-        <v>1500</v>
+        <v>185</v>
+      </c>
+      <c r="G233" s="2">
+        <v>25</v>
+      </c>
+      <c r="H233" s="2">
+        <v>91</v>
       </c>
       <c r="J233" s="6"/>
     </row>
@@ -14679,25 +14703,25 @@
         <v>11</v>
       </c>
       <c r="B234" s="6" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="C234" t="s">
         <v>125</v>
       </c>
       <c r="D234" s="10">
-        <v>45799</v>
+        <v>45792</v>
       </c>
       <c r="E234" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F234" s="6">
-        <v>417</v>
-      </c>
-      <c r="G234" s="6">
-        <v>65</v>
-      </c>
-      <c r="H234" s="6">
-        <v>1500</v>
+        <v>185</v>
+      </c>
+      <c r="G234" s="2">
+        <v>25</v>
+      </c>
+      <c r="H234" s="2">
+        <v>91</v>
       </c>
       <c r="I234" s="6" t="s">
         <v>88</v>
@@ -14709,25 +14733,25 @@
         <v>11</v>
       </c>
       <c r="B235" s="6" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="C235" t="s">
         <v>125</v>
       </c>
       <c r="D235" s="10">
-        <v>45944</v>
+        <v>45946</v>
       </c>
       <c r="E235" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F235" s="6">
-        <v>424</v>
+        <v>192</v>
       </c>
       <c r="G235" s="6">
-        <v>62</v>
+        <v>27</v>
       </c>
       <c r="H235" s="6">
-        <v>1530</v>
+        <v>109</v>
       </c>
       <c r="I235" s="6" t="s">
         <v>88</v>
@@ -14739,25 +14763,25 @@
         <v>11</v>
       </c>
       <c r="B236" s="6" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="C236" t="s">
         <v>125</v>
       </c>
       <c r="D236" s="10">
-        <v>45944</v>
+        <v>45945</v>
       </c>
       <c r="E236" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F236" s="6">
-        <v>34</v>
+        <v>201</v>
       </c>
       <c r="G236" s="6">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="H236" s="6">
-        <v>900</v>
+        <v>140</v>
       </c>
       <c r="I236" s="6" t="s">
         <v>88</v>
@@ -14765,29 +14789,32 @@
       <c r="J236" s="6"/>
     </row>
     <row r="237" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A237" t="s">
-        <v>11</v>
-      </c>
-      <c r="B237" t="s">
-        <v>12</v>
+      <c r="A237" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B237" s="6" t="s">
+        <v>81</v>
       </c>
       <c r="C237" t="s">
         <v>125</v>
       </c>
-      <c r="D237" s="1">
-        <v>45803</v>
-      </c>
-      <c r="E237" t="s">
+      <c r="D237" s="10">
+        <v>45946</v>
+      </c>
+      <c r="E237" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F237">
-        <v>398</v>
-      </c>
-      <c r="G237">
-        <v>55</v>
-      </c>
-      <c r="H237">
-        <v>1400</v>
+      <c r="F237" s="6">
+        <v>223</v>
+      </c>
+      <c r="G237" s="6">
+        <v>30</v>
+      </c>
+      <c r="H237" s="6">
+        <v>137</v>
+      </c>
+      <c r="I237" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="J237" s="6"/>
     </row>
@@ -14796,25 +14823,25 @@
         <v>11</v>
       </c>
       <c r="B238" s="6" t="s">
-        <v>12</v>
+        <v>77</v>
       </c>
       <c r="C238" t="s">
         <v>125</v>
       </c>
       <c r="D238" s="10">
-        <v>45803</v>
+        <v>45944</v>
       </c>
       <c r="E238" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F238" s="6">
-        <v>398</v>
+        <v>235</v>
       </c>
       <c r="G238" s="6">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="H238" s="6">
-        <v>1400</v>
+        <v>225</v>
       </c>
       <c r="I238" s="6" t="s">
         <v>88</v>
@@ -14822,29 +14849,32 @@
       <c r="J238" s="6"/>
     </row>
     <row r="239" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A239" t="s">
-        <v>11</v>
-      </c>
-      <c r="B239" t="s">
-        <v>12</v>
+      <c r="A239" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B239" s="6" t="s">
+        <v>75</v>
       </c>
       <c r="C239" t="s">
         <v>125</v>
       </c>
-      <c r="D239" s="1">
-        <v>45803</v>
-      </c>
-      <c r="E239" t="s">
+      <c r="D239" s="10">
+        <v>45946</v>
+      </c>
+      <c r="E239" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F239">
-        <v>383</v>
-      </c>
-      <c r="G239">
-        <v>50</v>
-      </c>
-      <c r="H239">
-        <v>940</v>
+      <c r="F239" s="6">
+        <v>240</v>
+      </c>
+      <c r="G239" s="6">
+        <v>30</v>
+      </c>
+      <c r="H239" s="6">
+        <v>219</v>
+      </c>
+      <c r="I239" s="6" t="s">
+        <v>88</v>
       </c>
       <c r="J239" s="6"/>
     </row>
@@ -14853,25 +14883,25 @@
         <v>11</v>
       </c>
       <c r="B240" s="6" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
       <c r="C240" t="s">
         <v>125</v>
       </c>
       <c r="D240" s="10">
-        <v>45803</v>
+        <v>45946</v>
       </c>
       <c r="E240" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F240" s="6">
-        <v>383</v>
+        <v>262</v>
       </c>
       <c r="G240" s="6">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H240" s="6">
-        <v>940</v>
+        <v>380</v>
       </c>
       <c r="I240" s="6" t="s">
         <v>88</v>
@@ -14883,25 +14913,25 @@
         <v>11</v>
       </c>
       <c r="B241" s="6" t="s">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="C241" t="s">
         <v>125</v>
       </c>
       <c r="D241" s="10">
-        <v>45946</v>
+        <v>45951</v>
       </c>
       <c r="E241" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F241" s="6">
-        <v>347</v>
+        <v>264</v>
       </c>
       <c r="G241" s="6">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="H241" s="6">
-        <v>990</v>
+        <v>300</v>
       </c>
       <c r="I241" s="6" t="s">
         <v>88</v>
@@ -14919,19 +14949,19 @@
         <v>125</v>
       </c>
       <c r="D242" s="10">
-        <v>45944</v>
+        <v>45946</v>
       </c>
       <c r="E242" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F242" s="6">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="G242" s="6">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H242" s="6">
-        <v>419</v>
+        <v>370</v>
       </c>
       <c r="I242" s="6" t="s">
         <v>88</v>
@@ -14943,25 +14973,25 @@
         <v>11</v>
       </c>
       <c r="B243" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C243" t="s">
         <v>125</v>
       </c>
       <c r="D243" s="10">
-        <v>45799</v>
+        <v>45944</v>
       </c>
       <c r="E243" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F243" s="6">
-        <v>155</v>
+        <v>285</v>
       </c>
       <c r="G243" s="6">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H243" s="6">
-        <v>150</v>
+        <v>419</v>
       </c>
       <c r="I243" s="6" t="s">
         <v>88</v>
@@ -14973,25 +15003,25 @@
         <v>11</v>
       </c>
       <c r="B244" s="6" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C244" t="s">
         <v>125</v>
       </c>
       <c r="D244" s="10">
-        <v>45944</v>
+        <v>45946</v>
       </c>
       <c r="E244" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F244" s="6">
-        <v>235</v>
+        <v>300</v>
       </c>
       <c r="G244" s="6">
         <v>40</v>
       </c>
       <c r="H244" s="6">
-        <v>225</v>
+        <v>550</v>
       </c>
       <c r="I244" s="6" t="s">
         <v>88</v>
@@ -15003,25 +15033,25 @@
         <v>11</v>
       </c>
       <c r="B245" s="6" t="s">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="C245" t="s">
         <v>125</v>
       </c>
       <c r="D245" s="10">
-        <v>45946</v>
+        <v>45944</v>
       </c>
       <c r="E245" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F245" s="6">
-        <v>283</v>
+        <v>340</v>
       </c>
       <c r="G245" s="6">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="H245" s="6">
-        <v>370</v>
+        <v>1250</v>
       </c>
       <c r="I245" s="6" t="s">
         <v>88</v>
@@ -15032,7 +15062,7 @@
         <v>11</v>
       </c>
       <c r="B246" s="6" t="s">
-        <v>81</v>
+        <v>51</v>
       </c>
       <c r="C246" t="s">
         <v>125</v>
@@ -15044,46 +15074,43 @@
         <v>21</v>
       </c>
       <c r="F246" s="6">
-        <v>262</v>
+        <v>347</v>
       </c>
       <c r="G246" s="6">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H246" s="6">
+        <v>990</v>
+      </c>
+      <c r="I246" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="J246" s="6"/>
+    </row>
+    <row r="247" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A247" t="s">
+        <v>11</v>
+      </c>
+      <c r="B247" t="s">
+        <v>51</v>
+      </c>
+      <c r="C247" t="s">
+        <v>125</v>
+      </c>
+      <c r="D247" s="1">
+        <v>45791</v>
+      </c>
+      <c r="E247" t="s">
+        <v>21</v>
+      </c>
+      <c r="F247">
         <v>380</v>
       </c>
-      <c r="I246" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="J246" s="6"/>
-    </row>
-    <row r="247" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A247" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B247" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="C247" t="s">
-        <v>125</v>
-      </c>
-      <c r="D247" s="10">
-        <v>45946</v>
-      </c>
-      <c r="E247" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F247" s="6">
-        <v>300</v>
-      </c>
-      <c r="G247" s="6">
-        <v>40</v>
-      </c>
-      <c r="H247" s="6">
-        <v>550</v>
-      </c>
-      <c r="I247" s="6" t="s">
-        <v>88</v>
+      <c r="G247">
+        <v>80</v>
+      </c>
+      <c r="H247">
+        <v>1450</v>
       </c>
     </row>
     <row r="248" spans="1:10" x14ac:dyDescent="0.35">
@@ -15091,25 +15118,25 @@
         <v>11</v>
       </c>
       <c r="B248" s="6" t="s">
-        <v>82</v>
+        <v>51</v>
       </c>
       <c r="C248" t="s">
         <v>125</v>
       </c>
       <c r="D248" s="10">
-        <v>45951</v>
+        <v>45791</v>
       </c>
       <c r="E248" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F248" s="6">
-        <v>264</v>
+        <v>380</v>
       </c>
       <c r="G248" s="6">
-        <v>35</v>
+        <v>80</v>
       </c>
       <c r="H248" s="6">
-        <v>300</v>
+        <v>1450</v>
       </c>
       <c r="I248" s="6" t="s">
         <v>88</v>
@@ -15117,32 +15144,29 @@
       <c r="J248" s="6"/>
     </row>
     <row r="249" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A249" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B249" s="6" t="s">
-        <v>75</v>
+      <c r="A249" t="s">
+        <v>11</v>
+      </c>
+      <c r="B249" t="s">
+        <v>12</v>
       </c>
       <c r="C249" t="s">
         <v>125</v>
       </c>
-      <c r="D249" s="10">
-        <v>45946</v>
-      </c>
-      <c r="E249" s="6" t="s">
+      <c r="D249" s="1">
+        <v>45803</v>
+      </c>
+      <c r="E249" t="s">
         <v>21</v>
       </c>
-      <c r="F249" s="6">
-        <v>240</v>
-      </c>
-      <c r="G249" s="6">
-        <v>30</v>
-      </c>
-      <c r="H249" s="6">
-        <v>219</v>
-      </c>
-      <c r="I249" s="6" t="s">
-        <v>88</v>
+      <c r="F249">
+        <v>383</v>
+      </c>
+      <c r="G249">
+        <v>50</v>
+      </c>
+      <c r="H249">
+        <v>940</v>
       </c>
     </row>
     <row r="250" spans="1:10" x14ac:dyDescent="0.35">
@@ -15150,25 +15174,25 @@
         <v>11</v>
       </c>
       <c r="B250" s="6" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
       <c r="C250" t="s">
         <v>125</v>
       </c>
       <c r="D250" s="10">
-        <v>45946</v>
+        <v>45803</v>
       </c>
       <c r="E250" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F250" s="6">
-        <v>223</v>
+        <v>383</v>
       </c>
       <c r="G250" s="6">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="H250" s="6">
-        <v>137</v>
+        <v>940</v>
       </c>
       <c r="I250" s="6" t="s">
         <v>88</v>
@@ -15176,32 +15200,29 @@
       <c r="J250" s="2"/>
     </row>
     <row r="251" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A251" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B251" s="6" t="s">
-        <v>102</v>
+      <c r="A251" t="s">
+        <v>11</v>
+      </c>
+      <c r="B251" t="s">
+        <v>12</v>
       </c>
       <c r="C251" t="s">
         <v>125</v>
       </c>
-      <c r="D251" s="10">
-        <v>45946</v>
-      </c>
-      <c r="E251" s="6" t="s">
+      <c r="D251" s="1">
+        <v>45803</v>
+      </c>
+      <c r="E251" t="s">
         <v>21</v>
       </c>
-      <c r="F251" s="6">
-        <v>192</v>
-      </c>
-      <c r="G251" s="6">
-        <v>27</v>
-      </c>
-      <c r="H251" s="6">
-        <v>109</v>
-      </c>
-      <c r="I251" s="6" t="s">
-        <v>88</v>
+      <c r="F251">
+        <v>398</v>
+      </c>
+      <c r="G251">
+        <v>55</v>
+      </c>
+      <c r="H251">
+        <v>1400</v>
       </c>
       <c r="J251" s="6"/>
     </row>
@@ -15210,25 +15231,25 @@
         <v>11</v>
       </c>
       <c r="B252" s="6" t="s">
-        <v>94</v>
+        <v>12</v>
       </c>
       <c r="C252" t="s">
         <v>125</v>
       </c>
       <c r="D252" s="10">
-        <v>45945</v>
+        <v>45803</v>
       </c>
       <c r="E252" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F252" s="6">
-        <v>201</v>
+        <v>398</v>
       </c>
       <c r="G252" s="6">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="H252" s="6">
-        <v>140</v>
+        <v>1400</v>
       </c>
       <c r="I252" s="6" t="s">
         <v>88</v>
@@ -15240,25 +15261,25 @@
         <v>11</v>
       </c>
       <c r="B253" t="s">
-        <v>81</v>
+        <v>45</v>
       </c>
       <c r="C253" t="s">
         <v>125</v>
       </c>
       <c r="D253" s="1">
-        <v>45792</v>
+        <v>45791</v>
       </c>
       <c r="E253" t="s">
         <v>21</v>
       </c>
       <c r="F253">
-        <v>185</v>
-      </c>
-      <c r="G253" s="2">
-        <v>25</v>
-      </c>
-      <c r="H253" s="2">
-        <v>91</v>
+        <v>405</v>
+      </c>
+      <c r="G253">
+        <v>76</v>
+      </c>
+      <c r="H253">
+        <v>1620</v>
       </c>
       <c r="J253" s="6"/>
     </row>
@@ -15267,57 +15288,57 @@
         <v>11</v>
       </c>
       <c r="B254" s="6" t="s">
-        <v>81</v>
+        <v>45</v>
       </c>
       <c r="C254" t="s">
         <v>125</v>
       </c>
       <c r="D254" s="10">
-        <v>45792</v>
+        <v>45791</v>
       </c>
       <c r="E254" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F254" s="6">
-        <v>185</v>
-      </c>
-      <c r="G254" s="2">
-        <v>25</v>
-      </c>
-      <c r="H254" s="2">
-        <v>91</v>
+        <v>405</v>
+      </c>
+      <c r="G254" s="6">
+        <v>76</v>
+      </c>
+      <c r="H254" s="6">
+        <v>1620</v>
       </c>
       <c r="I254" s="6" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="255" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A255" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B255" s="6" t="s">
-        <v>61</v>
+      <c r="A255" t="s">
+        <v>11</v>
+      </c>
+      <c r="B255" t="s">
+        <v>73</v>
       </c>
       <c r="C255" t="s">
         <v>125</v>
       </c>
-      <c r="D255" s="10">
-        <v>45944</v>
-      </c>
-      <c r="E255" s="6" t="s">
+      <c r="D255" s="1">
+        <v>45791</v>
+      </c>
+      <c r="E255" t="s">
         <v>21</v>
       </c>
-      <c r="F255" s="6">
-        <v>184</v>
-      </c>
-      <c r="G255" s="6">
-        <v>20</v>
-      </c>
-      <c r="H255" s="6">
-        <v>94</v>
-      </c>
-      <c r="I255" s="6" t="s">
-        <v>88</v>
+      <c r="F255">
+        <v>408</v>
+      </c>
+      <c r="G255">
+        <v>68</v>
+      </c>
+      <c r="H255">
+        <v>1470</v>
+      </c>
+      <c r="I255" t="s">
+        <v>74</v>
       </c>
       <c r="J255" s="6"/>
     </row>
@@ -15326,57 +15347,54 @@
         <v>11</v>
       </c>
       <c r="B256" s="6" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="C256" t="s">
         <v>125</v>
       </c>
       <c r="D256" s="10">
-        <v>45944</v>
+        <v>45791</v>
       </c>
       <c r="E256" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F256" s="6">
-        <v>156</v>
+        <v>408</v>
       </c>
       <c r="G256" s="6">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="H256" s="6">
-        <v>62</v>
+        <v>1470</v>
       </c>
       <c r="I256" s="6" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="257" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A257" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B257" s="6" t="s">
-        <v>92</v>
+      <c r="A257" t="s">
+        <v>11</v>
+      </c>
+      <c r="B257" t="s">
+        <v>12</v>
       </c>
       <c r="C257" t="s">
         <v>125</v>
       </c>
-      <c r="D257" s="10">
-        <v>45944</v>
-      </c>
-      <c r="E257" s="6" t="s">
+      <c r="D257" s="1">
+        <v>45803</v>
+      </c>
+      <c r="E257" t="s">
         <v>21</v>
       </c>
-      <c r="F257" s="6">
-        <v>156</v>
-      </c>
-      <c r="G257" s="6">
-        <v>20</v>
-      </c>
-      <c r="H257" s="6">
-        <v>57</v>
-      </c>
-      <c r="I257" s="6" t="s">
-        <v>88</v>
+      <c r="F257">
+        <v>414</v>
+      </c>
+      <c r="G257">
+        <v>70</v>
+      </c>
+      <c r="H257">
+        <v>1640</v>
       </c>
     </row>
     <row r="258" spans="1:10" x14ac:dyDescent="0.35">
@@ -15384,25 +15402,25 @@
         <v>11</v>
       </c>
       <c r="B258" s="6" t="s">
-        <v>92</v>
+        <v>12</v>
       </c>
       <c r="C258" t="s">
         <v>125</v>
       </c>
       <c r="D258" s="10">
-        <v>45945</v>
+        <v>45803</v>
       </c>
       <c r="E258" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F258" s="6">
-        <v>149</v>
+        <v>414</v>
       </c>
       <c r="G258" s="6">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="H258" s="6">
-        <v>50</v>
+        <v>1640</v>
       </c>
       <c r="I258" s="6" t="s">
         <v>88</v>
@@ -15413,25 +15431,25 @@
         <v>11</v>
       </c>
       <c r="B259" t="s">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="C259" t="s">
         <v>125</v>
       </c>
       <c r="D259" s="1">
-        <v>45803</v>
+        <v>45799</v>
       </c>
       <c r="E259" t="s">
         <v>21</v>
       </c>
       <c r="F259">
-        <v>145</v>
+        <v>417</v>
       </c>
       <c r="G259">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="H259">
-        <v>40</v>
+        <v>1500</v>
       </c>
       <c r="J259" s="6"/>
     </row>
@@ -15440,57 +15458,54 @@
         <v>11</v>
       </c>
       <c r="B260" s="6" t="s">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="C260" t="s">
         <v>125</v>
       </c>
       <c r="D260" s="10">
-        <v>45803</v>
+        <v>45799</v>
       </c>
       <c r="E260" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F260" s="6">
-        <v>145</v>
+        <v>417</v>
       </c>
       <c r="G260" s="6">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="H260" s="6">
-        <v>40</v>
+        <v>1500</v>
       </c>
       <c r="I260" s="6" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="261" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A261" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B261" s="6" t="s">
-        <v>93</v>
+      <c r="A261" t="s">
+        <v>11</v>
+      </c>
+      <c r="B261" t="s">
+        <v>45</v>
       </c>
       <c r="C261" t="s">
         <v>125</v>
       </c>
-      <c r="D261" s="10">
-        <v>45945</v>
-      </c>
-      <c r="E261" s="6" t="s">
+      <c r="D261" s="1">
+        <v>45791</v>
+      </c>
+      <c r="E261" t="s">
         <v>21</v>
       </c>
-      <c r="F261" s="6">
-        <v>106</v>
-      </c>
-      <c r="G261" s="6">
-        <v>18</v>
-      </c>
-      <c r="H261" s="6">
-        <v>10</v>
-      </c>
-      <c r="I261" s="6" t="s">
-        <v>88</v>
+      <c r="F261">
+        <v>424</v>
+      </c>
+      <c r="G261">
+        <v>76</v>
+      </c>
+      <c r="H261">
+        <v>1610</v>
       </c>
       <c r="J261" s="6"/>
     </row>
@@ -15499,25 +15514,25 @@
         <v>11</v>
       </c>
       <c r="B262" s="6" t="s">
-        <v>92</v>
+        <v>45</v>
       </c>
       <c r="C262" t="s">
         <v>125</v>
       </c>
       <c r="D262" s="10">
-        <v>45944</v>
+        <v>45791</v>
       </c>
       <c r="E262" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F262" s="6">
-        <v>148</v>
+        <v>424</v>
       </c>
       <c r="G262" s="6">
-        <v>15</v>
+        <v>76</v>
       </c>
       <c r="H262" s="6">
-        <v>52</v>
+        <v>1610</v>
       </c>
       <c r="I262" s="6" t="s">
         <v>88</v>
@@ -15541,13 +15556,13 @@
         <v>21</v>
       </c>
       <c r="F263" s="6">
-        <v>130</v>
+        <v>424</v>
       </c>
       <c r="G263" s="6">
-        <v>15</v>
+        <v>62</v>
       </c>
       <c r="H263" s="6">
-        <v>34</v>
+        <v>1530</v>
       </c>
       <c r="I263" s="6" t="s">
         <v>88</v>
@@ -15555,32 +15570,29 @@
       <c r="J263" s="6"/>
     </row>
     <row r="264" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A264" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B264" s="6" t="s">
-        <v>93</v>
+      <c r="A264" t="s">
+        <v>11</v>
+      </c>
+      <c r="B264" t="s">
+        <v>51</v>
       </c>
       <c r="C264" t="s">
         <v>125</v>
       </c>
-      <c r="D264" s="10">
-        <v>45944</v>
-      </c>
-      <c r="E264" s="6" t="s">
+      <c r="D264" s="1">
+        <v>45791</v>
+      </c>
+      <c r="E264" t="s">
         <v>21</v>
       </c>
-      <c r="F264" s="6">
-        <v>107</v>
-      </c>
-      <c r="G264" s="6">
-        <v>15</v>
-      </c>
-      <c r="H264" s="6">
-        <v>27</v>
-      </c>
-      <c r="I264" s="6" t="s">
-        <v>88</v>
+      <c r="F264">
+        <v>426</v>
+      </c>
+      <c r="G264">
+        <v>74</v>
+      </c>
+      <c r="H264">
+        <v>1700</v>
       </c>
       <c r="J264" s="6"/>
     </row>
@@ -15589,25 +15601,25 @@
         <v>11</v>
       </c>
       <c r="B265" s="6" t="s">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="C265" t="s">
         <v>125</v>
       </c>
       <c r="D265" s="10">
-        <v>45944</v>
+        <v>45791</v>
       </c>
       <c r="E265" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F265" s="6">
-        <v>106</v>
+        <v>426</v>
       </c>
       <c r="G265" s="6">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="H265" s="6">
-        <v>25</v>
+        <v>1700</v>
       </c>
       <c r="I265" s="6" t="s">
         <v>88</v>
@@ -15618,7 +15630,7 @@
         <v>11</v>
       </c>
       <c r="B266" t="s">
-        <v>79</v>
+        <v>12</v>
       </c>
       <c r="C266" t="s">
         <v>125</v>
@@ -15630,16 +15642,13 @@
         <v>21</v>
       </c>
       <c r="F266">
-        <v>155</v>
-      </c>
-      <c r="G266" s="2">
-        <v>15</v>
+        <v>435</v>
+      </c>
+      <c r="G266">
+        <v>70</v>
       </c>
       <c r="H266">
-        <v>41</v>
-      </c>
-      <c r="I266" t="s">
-        <v>80</v>
+        <v>1810</v>
       </c>
     </row>
     <row r="267" spans="1:10" x14ac:dyDescent="0.35">
@@ -15647,25 +15656,25 @@
         <v>11</v>
       </c>
       <c r="B267" s="6" t="s">
-        <v>92</v>
+        <v>12</v>
       </c>
       <c r="C267" t="s">
         <v>125</v>
       </c>
       <c r="D267" s="10">
-        <v>45944</v>
+        <v>45799</v>
       </c>
       <c r="E267" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F267" s="6">
-        <v>100</v>
+        <v>435</v>
       </c>
       <c r="G267" s="6">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="H267" s="6">
-        <v>15</v>
+        <v>1810</v>
       </c>
       <c r="I267" s="6" t="s">
         <v>88</v>
@@ -15673,61 +15682,58 @@
       <c r="J267" s="6"/>
     </row>
     <row r="268" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A268" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B268" s="6" t="s">
+      <c r="A268" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B268" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C268" t="s">
-        <v>125</v>
-      </c>
-      <c r="D268" s="10">
+      <c r="C268" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D268" s="11">
         <v>45944</v>
       </c>
-      <c r="E268" s="6" t="s">
+      <c r="E268" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F268" s="6">
-        <v>130</v>
-      </c>
-      <c r="G268" s="6">
-        <v>12</v>
-      </c>
-      <c r="H268" s="6">
-        <v>34</v>
-      </c>
-      <c r="I268" s="6" t="s">
+      <c r="F268" s="2">
+        <v>438</v>
+      </c>
+      <c r="G268" s="2">
+        <v>65</v>
+      </c>
+      <c r="H268" s="2">
+        <v>1670</v>
+      </c>
+      <c r="I268" s="2" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="269" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A269" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B269" s="6" t="s">
-        <v>93</v>
+      <c r="A269" t="s">
+        <v>11</v>
+      </c>
+      <c r="B269" t="s">
+        <v>55</v>
       </c>
       <c r="C269" t="s">
         <v>125</v>
       </c>
-      <c r="D269" s="10">
-        <v>45944</v>
-      </c>
-      <c r="E269" s="6" t="s">
+      <c r="D269" s="1">
+        <v>45799</v>
+      </c>
+      <c r="E269" t="s">
         <v>21</v>
       </c>
-      <c r="F269" s="6">
-        <v>107</v>
-      </c>
-      <c r="G269" s="6">
-        <v>12</v>
-      </c>
-      <c r="H269" s="6">
-        <v>17</v>
-      </c>
-      <c r="I269" s="6" t="s">
-        <v>88</v>
+      <c r="F269">
+        <v>450</v>
+      </c>
+      <c r="G269">
+        <v>70</v>
+      </c>
+      <c r="H269">
+        <v>2000</v>
       </c>
       <c r="J269" s="6" t="s">
         <v>74</v>
@@ -15738,57 +15744,54 @@
         <v>11</v>
       </c>
       <c r="B270" s="6" t="s">
-        <v>93</v>
+        <v>55</v>
       </c>
       <c r="C270" t="s">
         <v>125</v>
       </c>
       <c r="D270" s="10">
-        <v>45944</v>
+        <v>45799</v>
       </c>
       <c r="E270" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F270" s="6">
-        <v>126</v>
+        <v>450</v>
       </c>
       <c r="G270" s="6">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="H270" s="6">
-        <v>28</v>
+        <v>2000</v>
       </c>
       <c r="I270" s="6" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="271" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A271" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B271" s="6" t="s">
-        <v>93</v>
+      <c r="A271" t="s">
+        <v>11</v>
+      </c>
+      <c r="B271" t="s">
+        <v>55</v>
       </c>
       <c r="C271" t="s">
         <v>125</v>
       </c>
-      <c r="D271" s="10">
-        <v>45945</v>
-      </c>
-      <c r="E271" s="6" t="s">
+      <c r="D271" s="1">
+        <v>45791</v>
+      </c>
+      <c r="E271" t="s">
         <v>21</v>
       </c>
-      <c r="F271" s="6">
-        <v>123</v>
-      </c>
-      <c r="G271" s="6">
-        <v>10</v>
-      </c>
-      <c r="H271" s="6">
-        <v>25</v>
-      </c>
-      <c r="I271" s="6" t="s">
-        <v>88</v>
+      <c r="F271">
+        <v>458</v>
+      </c>
+      <c r="G271">
+        <v>68</v>
+      </c>
+      <c r="H271">
+        <v>1680</v>
       </c>
       <c r="J271" s="6"/>
     </row>
@@ -15797,58 +15800,58 @@
         <v>11</v>
       </c>
       <c r="B272" s="6" t="s">
-        <v>93</v>
+        <v>55</v>
       </c>
       <c r="C272" t="s">
         <v>125</v>
       </c>
       <c r="D272" s="10">
-        <v>45945</v>
+        <v>45791</v>
       </c>
       <c r="E272" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F272" s="6">
-        <v>112</v>
+        <v>458</v>
       </c>
       <c r="G272" s="6">
-        <v>10</v>
+        <v>68</v>
       </c>
       <c r="H272" s="6">
+        <v>1680</v>
+      </c>
+      <c r="I272" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="J272" s="6"/>
+    </row>
+    <row r="273" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A273" t="s">
+        <v>11</v>
+      </c>
+      <c r="B273" t="s">
+        <v>77</v>
+      </c>
+      <c r="C273" t="s">
+        <v>125</v>
+      </c>
+      <c r="D273" s="1">
+        <v>45803</v>
+      </c>
+      <c r="E273" t="s">
         <v>21</v>
       </c>
-      <c r="I272" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="J272" s="6"/>
-    </row>
-    <row r="273" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A273" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B273" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="C273" t="s">
-        <v>125</v>
-      </c>
-      <c r="D273" s="10">
-        <v>45945</v>
-      </c>
-      <c r="E273" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F273" s="6">
-        <v>102</v>
-      </c>
-      <c r="G273" s="6">
-        <v>10</v>
-      </c>
-      <c r="H273" s="6">
-        <v>16</v>
-      </c>
-      <c r="I273" s="6" t="s">
-        <v>88</v>
+      <c r="F273">
+        <v>463</v>
+      </c>
+      <c r="G273">
+        <v>80</v>
+      </c>
+      <c r="H273">
+        <v>2140</v>
+      </c>
+      <c r="I273" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="274" spans="1:10" x14ac:dyDescent="0.35">
@@ -15856,25 +15859,25 @@
         <v>11</v>
       </c>
       <c r="B274" s="6" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="C274" t="s">
         <v>125</v>
       </c>
       <c r="D274" s="10">
-        <v>45944</v>
+        <v>45803</v>
       </c>
       <c r="E274" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F274" s="6">
-        <v>96</v>
+        <v>463</v>
       </c>
       <c r="G274" s="6">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="H274" s="6">
-        <v>13</v>
+        <v>2140</v>
       </c>
       <c r="I274" s="6" t="s">
         <v>88</v>
@@ -15886,25 +15889,25 @@
         <v>11</v>
       </c>
       <c r="B275" s="6" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="C275" t="s">
         <v>125</v>
       </c>
       <c r="D275" s="10">
-        <v>45944</v>
+        <v>45946</v>
       </c>
       <c r="E275" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F275" s="6">
-        <v>99</v>
+        <v>465</v>
       </c>
       <c r="G275" s="6">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="H275" s="6">
-        <v>13</v>
+        <v>2430</v>
       </c>
       <c r="I275" s="6" t="s">
         <v>88</v>
@@ -15916,7 +15919,7 @@
         <v>11</v>
       </c>
       <c r="B276" s="6" t="s">
-        <v>93</v>
+        <v>61</v>
       </c>
       <c r="C276" t="s">
         <v>125</v>
@@ -15928,13 +15931,13 @@
         <v>21</v>
       </c>
       <c r="F276" s="6">
-        <v>92</v>
+        <v>470</v>
       </c>
       <c r="G276" s="6">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="H276" s="6">
-        <v>10</v>
+        <v>2480</v>
       </c>
       <c r="I276" s="6" t="s">
         <v>88</v>
@@ -15942,32 +15945,29 @@
       <c r="J276" s="6"/>
     </row>
     <row r="277" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A277" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B277" s="6" t="s">
-        <v>93</v>
+      <c r="A277" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B277" s="2" t="s">
+        <v>77</v>
       </c>
       <c r="C277" t="s">
         <v>125</v>
       </c>
-      <c r="D277" s="10">
-        <v>45944</v>
-      </c>
-      <c r="E277" s="6" t="s">
+      <c r="D277" s="11">
+        <v>45791</v>
+      </c>
+      <c r="E277" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F277" s="6">
-        <v>95</v>
-      </c>
-      <c r="G277" s="6">
-        <v>10</v>
-      </c>
-      <c r="H277" s="6">
-        <v>10</v>
-      </c>
-      <c r="I277" s="6" t="s">
-        <v>88</v>
+      <c r="F277" s="2">
+        <v>470</v>
+      </c>
+      <c r="G277" s="2">
+        <v>86</v>
+      </c>
+      <c r="H277" s="2">
+        <v>2460</v>
       </c>
       <c r="J277" s="6"/>
     </row>
@@ -15976,25 +15976,25 @@
         <v>11</v>
       </c>
       <c r="B278" s="6" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="C278" t="s">
         <v>125</v>
       </c>
       <c r="D278" s="10">
-        <v>45944</v>
+        <v>45791</v>
       </c>
       <c r="E278" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F278" s="6">
-        <v>92</v>
+        <v>470</v>
       </c>
       <c r="G278" s="6">
-        <v>10</v>
+        <v>86</v>
       </c>
       <c r="H278" s="6">
-        <v>12</v>
+        <v>2460</v>
       </c>
       <c r="I278" s="6" t="s">
         <v>88</v>
@@ -16005,25 +16005,25 @@
         <v>11</v>
       </c>
       <c r="B279" s="6" t="s">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="C279" t="s">
         <v>125</v>
       </c>
       <c r="D279" s="10">
-        <v>45944</v>
+        <v>45951</v>
       </c>
       <c r="E279" s="6" t="s">
         <v>21</v>
       </c>
       <c r="F279" s="6">
-        <v>86</v>
+        <v>494</v>
       </c>
       <c r="G279" s="6">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="H279" s="6">
-        <v>10</v>
+        <v>2390</v>
       </c>
       <c r="I279" s="6" t="s">
         <v>88</v>
@@ -22059,6 +22059,11 @@
       <c r="J486" s="6"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I486" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I486">
+      <sortCondition ref="E1:E486"/>
+    </sortState>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J487">
     <sortCondition ref="H1:H487"/>
   </sortState>
@@ -28060,6 +28065,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="7ce4cce1-0673-44d6-a8e9-024984c6c156" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010008813DEC4A17DB40A5843D1157D8CD4D" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dc6577e42519716f75255cf7493b32f7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9" xmlns:ns3="7ce4cce1-0673-44d6-a8e9-024984c6c156" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="93d8227084f1dc13f4d26d22ce1da744" ns2:_="" ns3:_="">
     <xsd:import namespace="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9"/>
@@ -28314,17 +28330,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="7ce4cce1-0673-44d6-a8e9-024984c6c156" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -28335,6 +28340,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C3512AB9-A13E-4245-B2A0-964E627FDE40}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="7ce4cce1-0673-44d6-a8e9-024984c6c156"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3258F12-C15B-4654-A491-0335704C572D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -28353,23 +28375,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C3512AB9-A13E-4245-B2A0-964E627FDE40}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="7ce4cce1-0673-44d6-a8e9-024984c6c156"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0785BFC6-745B-49B0-87B9-892A72BBB88F}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Fixed Bin width and FL by Mass plots
Renamed bin‑width variable to BIN_WIDTH_CM for correct units and updated the FL by Mass plot to use a log‑x fit to better match the observed data pattern
</commit_message>
<xml_diff>
--- a/01_data/01_raw_files/Fixed_fish_widths_DraftExcelAnalysis_Feb2026.xlsx
+++ b/01_data/01_raw_files/Fixed_fish_widths_DraftExcelAnalysis_Feb2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RIZZUTOM\Desktop\GitHub Projects\2026_Reddick_fish_morphology\01_data\01_raw_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA90AB9B-31BF-4537-8A59-279C1D8762AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FCB0946-BBB1-4D6F-98AE-606D02CE2283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13544,31 +13544,31 @@
       <c r="J194" s="6"/>
     </row>
     <row r="195" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A195" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B195" s="6" t="s">
+      <c r="A195" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B195" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="C195" t="s">
-        <v>125</v>
-      </c>
-      <c r="D195" s="10">
+      <c r="C195" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D195" s="11">
         <v>45945</v>
       </c>
-      <c r="E195" s="6" t="s">
+      <c r="E195" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F195" s="6">
+      <c r="F195" s="2">
         <v>750</v>
       </c>
-      <c r="G195" s="6">
+      <c r="G195" s="2">
         <v>40</v>
       </c>
-      <c r="H195" s="6">
+      <c r="H195" s="2">
         <v>370</v>
       </c>
-      <c r="I195" s="6" t="s">
+      <c r="I195" s="2" t="s">
         <v>88</v>
       </c>
     </row>
@@ -28060,17 +28060,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="7ce4cce1-0673-44d6-a8e9-024984c6c156" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010008813DEC4A17DB40A5843D1157D8CD4D" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dc6577e42519716f75255cf7493b32f7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9" xmlns:ns3="7ce4cce1-0673-44d6-a8e9-024984c6c156" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="93d8227084f1dc13f4d26d22ce1da744" ns2:_="" ns3:_="">
     <xsd:import namespace="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9"/>
@@ -28325,6 +28314,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="7ce4cce1-0673-44d6-a8e9-024984c6c156" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -28335,23 +28335,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C3512AB9-A13E-4245-B2A0-964E627FDE40}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="7ce4cce1-0673-44d6-a8e9-024984c6c156"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3258F12-C15B-4654-A491-0335704C572D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -28370,6 +28353,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C3512AB9-A13E-4245-B2A0-964E627FDE40}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="7ce4cce1-0673-44d6-a8e9-024984c6c156"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0785BFC6-745B-49B0-87B9-892A72BBB88F}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
v1.22 added results table + patchwork edits
Added results table and quality edits to the patchwork plots
</commit_message>
<xml_diff>
--- a/01_data/01_raw_files/Fixed_fish_widths_DraftExcelAnalysis_Feb2026.xlsx
+++ b/01_data/01_raw_files/Fixed_fish_widths_DraftExcelAnalysis_Feb2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RIZZUTOM\Desktop\GitHub Projects\2026_Reddick_fish_morphology\01_data\01_raw_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C9FE061-19E4-4C24-9BB0-E05B5B7DB052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05ADED76-59D3-4CC3-9A91-89F50073B927}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -533,16 +533,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF00B0F0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -646,18 +637,180 @@
               <c:f>Sheet1!$F$2:$F$63</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="62"/>
                 <c:pt idx="0">
+                  <c:v>220</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>370</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>185</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>172</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>160</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>193</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>186</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>84</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>217</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>208</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>179</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>77</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>94</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>93</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>241</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>226</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>183</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>400</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>395</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>115</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>192</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>180</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>93</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>94</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>91</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>142</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>683</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>123</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>380</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>326</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>349</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>596</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>175</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>174</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>290</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>286</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>279</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>280</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>266</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>271</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>119</c:v>
+                </c:pt>
+                <c:pt idx="51">
                   <c:v>86</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="52">
                   <c:v>126</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="53">
                   <c:v>123</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="54">
                   <c:v>112</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>51</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>106</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>83</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>78</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>192</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>186</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -667,18 +820,180 @@
               <c:f>Sheet1!$G$2:$G$63</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="62"/>
                 <c:pt idx="0">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="13">
                   <c:v>8</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="14">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>55</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>83</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>66</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>59</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>57</c:v>
+                </c:pt>
+                <c:pt idx="50">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="51">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="52">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="53">
                   <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>26</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7002,7 +7317,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AH485"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -7054,7 +7368,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>11</v>
       </c>
@@ -7087,7 +7401,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>11</v>
       </c>
@@ -7120,7 +7434,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
         <v>11</v>
       </c>
@@ -7155,7 +7469,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>11</v>
       </c>
@@ -7190,7 +7504,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
         <v>11</v>
       </c>
@@ -7223,7 +7537,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
         <v>11</v>
       </c>
@@ -7256,7 +7570,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="15" t="s">
         <v>11</v>
       </c>
@@ -7289,7 +7603,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="9" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
         <v>11</v>
       </c>
@@ -7324,7 +7638,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>11</v>
       </c>
@@ -7353,7 +7667,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
         <v>11</v>
       </c>
@@ -7386,7 +7700,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
         <v>11</v>
       </c>
@@ -7419,7 +7733,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
         <v>11</v>
       </c>
@@ -7451,7 +7765,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -7484,7 +7798,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
         <v>11</v>
       </c>
@@ -7517,7 +7831,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="16" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
         <v>11</v>
       </c>
@@ -7550,7 +7864,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="17" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A17" s="6" t="s">
         <v>11</v>
       </c>
@@ -7583,7 +7897,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
         <v>11</v>
       </c>
@@ -7616,7 +7930,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
         <v>11</v>
       </c>
@@ -7649,7 +7963,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A20" s="6" t="s">
         <v>11</v>
       </c>
@@ -7682,7 +7996,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
         <v>11</v>
       </c>
@@ -7715,7 +8029,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="22" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A22" s="13" t="s">
         <v>11</v>
       </c>
@@ -7748,7 +8062,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A23" s="6" t="s">
         <v>11</v>
       </c>
@@ -7781,7 +8095,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A24" s="6" t="s">
         <v>11</v>
       </c>
@@ -7814,7 +8128,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A25" s="6" t="s">
         <v>11</v>
       </c>
@@ -7844,7 +8158,7 @@
       </c>
       <c r="J25" s="6"/>
     </row>
-    <row r="26" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A26" s="6" t="s">
         <v>11</v>
       </c>
@@ -7877,7 +8191,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="27" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A27" s="6" t="s">
         <v>11</v>
       </c>
@@ -7921,7 +8235,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="28" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>11</v>
       </c>
@@ -7966,7 +8280,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="29" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>11</v>
       </c>
@@ -8011,7 +8325,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>11</v>
       </c>
@@ -8056,7 +8370,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A31" s="6" t="s">
         <v>11</v>
       </c>
@@ -8097,7 +8411,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="32" spans="1:34" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="6" t="s">
         <v>11</v>
       </c>
@@ -8157,7 +8471,7 @@
       <c r="AG32"/>
       <c r="AH32"/>
     </row>
-    <row r="33" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A33" s="6" t="s">
         <v>11</v>
       </c>
@@ -8202,7 +8516,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="34" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A34" s="6" t="s">
         <v>11</v>
       </c>
@@ -8247,7 +8561,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A35" s="6" t="s">
         <v>11</v>
       </c>
@@ -8292,7 +8606,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="36" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A36" s="6" t="s">
         <v>11</v>
       </c>
@@ -8337,7 +8651,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A37" s="6" t="s">
         <v>11</v>
       </c>
@@ -8378,7 +8692,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="38" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A38" s="6" t="s">
         <v>11</v>
       </c>
@@ -8423,7 +8737,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="39" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A39" s="6" t="s">
         <v>11</v>
       </c>
@@ -8468,7 +8782,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="40" spans="1:34" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="6" t="s">
         <v>11</v>
       </c>
@@ -8525,7 +8839,7 @@
       <c r="AG40"/>
       <c r="AH40"/>
     </row>
-    <row r="41" spans="1:34" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="6" t="s">
         <v>11</v>
       </c>
@@ -8582,37 +8896,37 @@
       <c r="AG41"/>
       <c r="AH41"/>
     </row>
-    <row r="42" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>11</v>
-      </c>
-      <c r="B42" t="s">
+    <row r="42" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="A42" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B42" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="C42" t="s">
-        <v>125</v>
-      </c>
-      <c r="D42" s="1">
+      <c r="C42" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="D42" s="14">
         <v>46361</v>
       </c>
-      <c r="E42" t="s">
+      <c r="E42" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="F42">
+      <c r="F42" s="13">
         <v>596</v>
       </c>
-      <c r="G42">
+      <c r="G42" s="13">
         <v>83</v>
       </c>
-      <c r="H42">
-        <v>510</v>
-      </c>
-      <c r="I42" s="6" t="s">
+      <c r="H42" s="13">
+        <v>2510</v>
+      </c>
+      <c r="I42" s="13" t="s">
         <v>88</v>
       </c>
       <c r="J42" s="6"/>
     </row>
-    <row r="43" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A43" s="6" t="s">
         <v>11</v>
       </c>
@@ -8642,7 +8956,7 @@
       </c>
       <c r="J43" s="6"/>
     </row>
-    <row r="44" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A44" s="6" t="s">
         <v>11</v>
       </c>
@@ -8672,7 +8986,7 @@
       </c>
       <c r="J44" s="6"/>
     </row>
-    <row r="45" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A45" s="6" t="s">
         <v>11</v>
       </c>
@@ -8702,7 +9016,7 @@
       </c>
       <c r="J45" s="6"/>
     </row>
-    <row r="46" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>4</v>
       </c>
@@ -8732,7 +9046,7 @@
       </c>
       <c r="J46" s="6"/>
     </row>
-    <row r="47" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>4</v>
       </c>
@@ -8762,7 +9076,7 @@
       </c>
       <c r="J47" s="6"/>
     </row>
-    <row r="48" spans="1:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:34" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>4</v>
       </c>
@@ -8792,7 +9106,7 @@
       </c>
       <c r="J48" s="6"/>
     </row>
-    <row r="49" spans="1:10" s="2" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>4</v>
       </c>
@@ -8822,7 +9136,7 @@
       </c>
       <c r="J49" s="6"/>
     </row>
-    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>4</v>
       </c>
@@ -8852,7 +9166,7 @@
       </c>
       <c r="J50" s="6"/>
     </row>
-    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>4</v>
       </c>
@@ -8882,7 +9196,7 @@
       </c>
       <c r="J51" s="6"/>
     </row>
-    <row r="52" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" s="6" t="s">
         <v>11</v>
       </c>
@@ -9031,7 +9345,7 @@
       </c>
       <c r="J56" s="6"/>
     </row>
-    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" s="6" t="s">
         <v>11</v>
       </c>
@@ -9061,7 +9375,7 @@
       </c>
       <c r="J57" s="6"/>
     </row>
-    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" s="6" t="s">
         <v>11</v>
       </c>
@@ -9091,7 +9405,7 @@
       </c>
       <c r="J58" s="6"/>
     </row>
-    <row r="59" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" s="6" t="s">
         <v>11</v>
       </c>
@@ -9121,7 +9435,7 @@
       </c>
       <c r="J59" s="6"/>
     </row>
-    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" s="6" t="s">
         <v>11</v>
       </c>
@@ -9151,7 +9465,7 @@
       </c>
       <c r="J60" s="6"/>
     </row>
-    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" s="6" t="s">
         <v>11</v>
       </c>
@@ -9181,7 +9495,7 @@
       </c>
       <c r="J61" s="6"/>
     </row>
-    <row r="62" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" s="6" t="s">
         <v>11</v>
       </c>
@@ -9211,7 +9525,7 @@
       </c>
       <c r="J62" s="6"/>
     </row>
-    <row r="63" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" s="6" t="s">
         <v>11</v>
       </c>
@@ -9241,7 +9555,7 @@
       </c>
       <c r="J63" s="6"/>
     </row>
-    <row r="64" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" s="6" t="s">
         <v>11</v>
       </c>
@@ -9271,7 +9585,7 @@
       </c>
       <c r="J64" s="6"/>
     </row>
-    <row r="65" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" s="13" t="s">
         <v>11</v>
       </c>
@@ -9297,7 +9611,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66" s="6" t="s">
         <v>11</v>
       </c>
@@ -9327,7 +9641,7 @@
       </c>
       <c r="J66" s="6"/>
     </row>
-    <row r="67" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" s="6" t="s">
         <v>11</v>
       </c>
@@ -9357,7 +9671,7 @@
       </c>
       <c r="J67" s="6"/>
     </row>
-    <row r="68" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" s="6" t="s">
         <v>11</v>
       </c>
@@ -9387,7 +9701,7 @@
       </c>
       <c r="J68" s="6"/>
     </row>
-    <row r="69" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" s="6" t="s">
         <v>11</v>
       </c>
@@ -9413,7 +9727,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="70" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70" s="6" t="s">
         <v>11</v>
       </c>
@@ -9443,7 +9757,7 @@
       </c>
       <c r="J70" s="6"/>
     </row>
-    <row r="71" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" s="6" t="s">
         <v>11</v>
       </c>
@@ -9473,7 +9787,7 @@
       </c>
       <c r="J71" s="6"/>
     </row>
-    <row r="72" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72" s="6" t="s">
         <v>11</v>
       </c>
@@ -9503,7 +9817,7 @@
       </c>
       <c r="J72" s="6"/>
     </row>
-    <row r="73" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" s="6" t="s">
         <v>11</v>
       </c>
@@ -9533,7 +9847,7 @@
       </c>
       <c r="J73" s="6"/>
     </row>
-    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A74" s="6" t="s">
         <v>11</v>
       </c>
@@ -9563,7 +9877,7 @@
       </c>
       <c r="J74" s="6"/>
     </row>
-    <row r="75" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A75" s="6" t="s">
         <v>11</v>
       </c>
@@ -9593,7 +9907,7 @@
       </c>
       <c r="J75" s="6"/>
     </row>
-    <row r="76" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A76" s="6" t="s">
         <v>11</v>
       </c>
@@ -9623,7 +9937,7 @@
       </c>
       <c r="J76" s="6"/>
     </row>
-    <row r="77" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A77" s="6" t="s">
         <v>11</v>
       </c>
@@ -9653,7 +9967,7 @@
       </c>
       <c r="J77" s="6"/>
     </row>
-    <row r="78" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A78" s="6" t="s">
         <v>11</v>
       </c>
@@ -9682,7 +9996,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="79" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A79" s="6" t="s">
         <v>11</v>
       </c>
@@ -9712,7 +10026,7 @@
       </c>
       <c r="J79" s="6"/>
     </row>
-    <row r="80" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A80" s="6" t="s">
         <v>11</v>
       </c>
@@ -9741,7 +10055,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="81" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A81" s="6" t="s">
         <v>11</v>
       </c>
@@ -9771,7 +10085,7 @@
       </c>
       <c r="J81" s="6"/>
     </row>
-    <row r="82" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A82" s="6" t="s">
         <v>11</v>
       </c>
@@ -9800,7 +10114,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="83" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>4</v>
       </c>
@@ -9829,7 +10143,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="84" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>4</v>
       </c>
@@ -9859,7 +10173,7 @@
       </c>
       <c r="J84" s="6"/>
     </row>
-    <row r="85" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>4</v>
       </c>
@@ -9889,7 +10203,7 @@
       </c>
       <c r="J85" s="6"/>
     </row>
-    <row r="86" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>4</v>
       </c>
@@ -9919,7 +10233,7 @@
       </c>
       <c r="J86" s="6"/>
     </row>
-    <row r="87" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A87" s="6" t="s">
         <v>4</v>
       </c>
@@ -9948,7 +10262,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="88" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>4</v>
       </c>
@@ -9980,7 +10294,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="89" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A89" s="6" t="s">
         <v>11</v>
       </c>
@@ -10575,7 +10889,7 @@
       </c>
       <c r="J108" s="6"/>
     </row>
-    <row r="109" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" s="6" t="s">
         <v>11</v>
       </c>
@@ -10605,7 +10919,7 @@
       </c>
       <c r="J109" s="6"/>
     </row>
-    <row r="110" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" s="6" t="s">
         <v>11</v>
       </c>
@@ -10635,7 +10949,7 @@
       </c>
       <c r="J110" s="6"/>
     </row>
-    <row r="111" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A111" s="6" t="s">
         <v>11</v>
       </c>
@@ -10665,7 +10979,7 @@
       </c>
       <c r="J111" s="6"/>
     </row>
-    <row r="112" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A112" s="6" t="s">
         <v>11</v>
       </c>
@@ -10695,7 +11009,7 @@
       </c>
       <c r="J112" s="6"/>
     </row>
-    <row r="113" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A113" s="6" t="s">
         <v>11</v>
       </c>
@@ -10725,7 +11039,7 @@
       </c>
       <c r="J113" s="6"/>
     </row>
-    <row r="114" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A114" s="6" t="s">
         <v>11</v>
       </c>
@@ -10755,7 +11069,7 @@
       </c>
       <c r="J114" s="6"/>
     </row>
-    <row r="115" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A115" s="6" t="s">
         <v>11</v>
       </c>
@@ -10785,7 +11099,7 @@
       </c>
       <c r="J115" s="6"/>
     </row>
-    <row r="116" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A116" s="6" t="s">
         <v>11</v>
       </c>
@@ -10815,7 +11129,7 @@
       </c>
       <c r="J116" s="6"/>
     </row>
-    <row r="117" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A117" s="6" t="s">
         <v>11</v>
       </c>
@@ -10844,7 +11158,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="118" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A118" s="6" t="s">
         <v>11</v>
       </c>
@@ -10873,7 +11187,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="119" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A119" s="13" t="s">
         <v>11</v>
       </c>
@@ -10903,7 +11217,7 @@
       </c>
       <c r="J119" s="6"/>
     </row>
-    <row r="120" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A120" s="6" t="s">
         <v>11</v>
       </c>
@@ -10933,7 +11247,7 @@
       </c>
       <c r="J120" s="6"/>
     </row>
-    <row r="121" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A121" s="6" t="s">
         <v>11</v>
       </c>
@@ -10963,7 +11277,7 @@
       </c>
       <c r="J121" s="6"/>
     </row>
-    <row r="122" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A122" s="6" t="s">
         <v>11</v>
       </c>
@@ -10992,7 +11306,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="123" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A123" s="6" t="s">
         <v>11</v>
       </c>
@@ -11022,7 +11336,7 @@
       </c>
       <c r="J123" s="6"/>
     </row>
-    <row r="124" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A124" s="6" t="s">
         <v>11</v>
       </c>
@@ -11051,7 +11365,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="125" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A125" s="6" t="s">
         <v>11</v>
       </c>
@@ -11081,7 +11395,7 @@
       </c>
       <c r="J125" s="6"/>
     </row>
-    <row r="126" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A126" s="6" t="s">
         <v>11</v>
       </c>
@@ -11110,7 +11424,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="127" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A127" s="6" t="s">
         <v>11</v>
       </c>
@@ -11140,7 +11454,7 @@
       </c>
       <c r="J127" s="6"/>
     </row>
-    <row r="128" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A128" s="6" t="s">
         <v>11</v>
       </c>
@@ -11170,7 +11484,7 @@
       </c>
       <c r="J128" s="6"/>
     </row>
-    <row r="129" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A129" s="6" t="s">
         <v>11</v>
       </c>
@@ -11200,7 +11514,7 @@
       </c>
       <c r="J129" s="6"/>
     </row>
-    <row r="130" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>11</v>
       </c>
@@ -11230,7 +11544,7 @@
       </c>
       <c r="J130" s="6"/>
     </row>
-    <row r="131" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A131" s="6" t="s">
         <v>11</v>
       </c>
@@ -11260,7 +11574,7 @@
       </c>
       <c r="J131" s="6"/>
     </row>
-    <row r="132" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A132" s="6" t="s">
         <v>11</v>
       </c>
@@ -11290,7 +11604,7 @@
       </c>
       <c r="J132" s="6"/>
     </row>
-    <row r="133" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A133" s="6" t="s">
         <v>11</v>
       </c>
@@ -11320,7 +11634,7 @@
       </c>
       <c r="J133" s="6"/>
     </row>
-    <row r="134" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A134" s="6" t="s">
         <v>11</v>
       </c>
@@ -11349,7 +11663,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="135" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A135" s="6" t="s">
         <v>11</v>
       </c>
@@ -11379,7 +11693,7 @@
       </c>
       <c r="J135" s="6"/>
     </row>
-    <row r="136" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A136" s="6" t="s">
         <v>11</v>
       </c>
@@ -11409,7 +11723,7 @@
       </c>
       <c r="J136" s="6"/>
     </row>
-    <row r="137" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A137" s="13" t="s">
         <v>11</v>
       </c>
@@ -11439,7 +11753,7 @@
       </c>
       <c r="J137" s="6"/>
     </row>
-    <row r="138" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A138" s="6" t="s">
         <v>11</v>
       </c>
@@ -11469,7 +11783,7 @@
       </c>
       <c r="J138" s="6"/>
     </row>
-    <row r="139" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>4</v>
       </c>
@@ -11499,7 +11813,7 @@
       </c>
       <c r="J139" s="6"/>
     </row>
-    <row r="140" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A140" s="6" t="s">
         <v>11</v>
       </c>
@@ -11529,7 +11843,7 @@
       </c>
       <c r="J140" s="6"/>
     </row>
-    <row r="141" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A141" s="6" t="s">
         <v>11</v>
       </c>
@@ -11559,7 +11873,7 @@
       </c>
       <c r="J141" s="6"/>
     </row>
-    <row r="142" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A142" s="6" t="s">
         <v>11</v>
       </c>
@@ -11585,7 +11899,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="143" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A143" s="6" t="s">
         <v>11</v>
       </c>
@@ -11615,7 +11929,7 @@
       </c>
       <c r="J143" s="6"/>
     </row>
-    <row r="144" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A144" s="6" t="s">
         <v>11</v>
       </c>
@@ -11645,7 +11959,7 @@
       </c>
       <c r="J144" s="6"/>
     </row>
-    <row r="145" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A145" s="6" t="s">
         <v>11</v>
       </c>
@@ -11674,7 +11988,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="146" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A146" s="6" t="s">
         <v>11</v>
       </c>
@@ -11704,7 +12018,7 @@
       </c>
       <c r="J146" s="6"/>
     </row>
-    <row r="147" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A147" s="6" t="s">
         <v>11</v>
       </c>
@@ -11734,7 +12048,7 @@
       </c>
       <c r="J147" s="6"/>
     </row>
-    <row r="148" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A148" s="6" t="s">
         <v>11</v>
       </c>
@@ -11764,7 +12078,7 @@
       </c>
       <c r="J148" s="6"/>
     </row>
-    <row r="149" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A149" s="6" t="s">
         <v>11</v>
       </c>
@@ -11794,7 +12108,7 @@
       </c>
       <c r="J149" s="6"/>
     </row>
-    <row r="150" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A150" s="6" t="s">
         <v>11</v>
       </c>
@@ -11824,7 +12138,7 @@
       </c>
       <c r="J150" s="6"/>
     </row>
-    <row r="151" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>11</v>
       </c>
@@ -11854,7 +12168,7 @@
       </c>
       <c r="J151" s="6"/>
     </row>
-    <row r="152" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>4</v>
       </c>
@@ -11974,7 +12288,7 @@
       </c>
       <c r="J155" s="6"/>
     </row>
-    <row r="156" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>11</v>
       </c>
@@ -12004,7 +12318,7 @@
       </c>
       <c r="J156" s="6"/>
     </row>
-    <row r="157" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A157" s="6" t="s">
         <v>11</v>
       </c>
@@ -12033,7 +12347,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="158" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A158" s="6" t="s">
         <v>11</v>
       </c>
@@ -12063,7 +12377,7 @@
       </c>
       <c r="J158" s="6"/>
     </row>
-    <row r="159" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A159" s="6" t="s">
         <v>11</v>
       </c>
@@ -12092,7 +12406,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="160" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A160" s="6" t="s">
         <v>11</v>
       </c>
@@ -12121,7 +12435,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="161" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A161" s="6" t="s">
         <v>11</v>
       </c>
@@ -12151,7 +12465,7 @@
       </c>
       <c r="J161" s="6"/>
     </row>
-    <row r="162" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A162" s="6" t="s">
         <v>11</v>
       </c>
@@ -12181,7 +12495,7 @@
       </c>
       <c r="J162" s="6"/>
     </row>
-    <row r="163" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A163" s="6" t="s">
         <v>11</v>
       </c>
@@ -12211,7 +12525,7 @@
       </c>
       <c r="J163" s="6"/>
     </row>
-    <row r="164" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A164" s="6" t="s">
         <v>11</v>
       </c>
@@ -12240,7 +12554,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="165" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>4</v>
       </c>
@@ -12270,7 +12584,7 @@
       </c>
       <c r="J165" s="6"/>
     </row>
-    <row r="166" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>4</v>
       </c>
@@ -12300,7 +12614,7 @@
       </c>
       <c r="J166" s="6"/>
     </row>
-    <row r="167" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A167" s="6" t="s">
         <v>4</v>
       </c>
@@ -12329,7 +12643,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="168" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A168" s="6" t="s">
         <v>11</v>
       </c>
@@ -12388,7 +12702,7 @@
       </c>
       <c r="J169" s="6"/>
     </row>
-    <row r="170" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>11</v>
       </c>
@@ -12418,7 +12732,7 @@
       </c>
       <c r="J170" s="6"/>
     </row>
-    <row r="171" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A171" s="6" t="s">
         <v>11</v>
       </c>
@@ -12447,7 +12761,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="172" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A172" s="2" t="s">
         <v>11</v>
       </c>
@@ -12476,7 +12790,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="173" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>11</v>
       </c>
@@ -12506,7 +12820,7 @@
       </c>
       <c r="J173" s="6"/>
     </row>
-    <row r="174" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>4</v>
       </c>
@@ -12535,7 +12849,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="175" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A175" s="6" t="s">
         <v>11</v>
       </c>
@@ -12564,7 +12878,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="176" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>11</v>
       </c>
@@ -12594,7 +12908,7 @@
       </c>
       <c r="J176" s="6"/>
     </row>
-    <row r="177" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>4</v>
       </c>
@@ -12623,7 +12937,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="178" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>4</v>
       </c>
@@ -12653,7 +12967,7 @@
       </c>
       <c r="J178" s="6"/>
     </row>
-    <row r="179" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>4</v>
       </c>
@@ -12682,7 +12996,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="180" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A180" s="6" t="s">
         <v>11</v>
       </c>
@@ -12712,7 +13026,7 @@
       </c>
       <c r="J180" s="6"/>
     </row>
-    <row r="181" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A181" s="6" t="s">
         <v>11</v>
       </c>
@@ -12741,7 +13055,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="182" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>11</v>
       </c>
@@ -12771,7 +13085,7 @@
       </c>
       <c r="J182" s="6"/>
     </row>
-    <row r="183" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>11</v>
       </c>
@@ -12801,7 +13115,7 @@
       </c>
       <c r="J183" s="6"/>
     </row>
-    <row r="184" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>11</v>
       </c>
@@ -12831,7 +13145,7 @@
       </c>
       <c r="J184" s="6"/>
     </row>
-    <row r="185" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>11</v>
       </c>
@@ -12861,7 +13175,7 @@
       </c>
       <c r="J185" s="6"/>
     </row>
-    <row r="186" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A186" s="6" t="s">
         <v>11</v>
       </c>
@@ -12891,7 +13205,7 @@
       </c>
       <c r="J186" s="6"/>
     </row>
-    <row r="187" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A187" s="6" t="s">
         <v>11</v>
       </c>
@@ -12921,7 +13235,7 @@
       </c>
       <c r="J187" s="6"/>
     </row>
-    <row r="188" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>11</v>
       </c>
@@ -12951,7 +13265,7 @@
       </c>
       <c r="J188" s="6"/>
     </row>
-    <row r="189" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A189" s="6" t="s">
         <v>11</v>
       </c>
@@ -12981,7 +13295,7 @@
       </c>
       <c r="J189" s="6"/>
     </row>
-    <row r="190" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A190" s="6" t="s">
         <v>11</v>
       </c>
@@ -13011,7 +13325,7 @@
       </c>
       <c r="J190" s="6"/>
     </row>
-    <row r="191" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A191" s="6" t="s">
         <v>11</v>
       </c>
@@ -13041,7 +13355,7 @@
       </c>
       <c r="J191" s="6"/>
     </row>
-    <row r="192" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>11</v>
       </c>
@@ -13068,7 +13382,7 @@
       </c>
       <c r="J192" s="6"/>
     </row>
-    <row r="193" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A193" s="6" t="s">
         <v>11</v>
       </c>
@@ -13097,7 +13411,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="194" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A194" s="6" t="s">
         <v>11</v>
       </c>
@@ -13127,7 +13441,7 @@
       </c>
       <c r="J194" s="6"/>
     </row>
-    <row r="195" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A195" s="6" t="s">
         <v>11</v>
       </c>
@@ -13156,7 +13470,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="196" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A196" s="6" t="s">
         <v>11</v>
       </c>
@@ -13186,7 +13500,7 @@
       </c>
       <c r="J196" s="6"/>
     </row>
-    <row r="197" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A197" s="6" t="s">
         <v>11</v>
       </c>
@@ -13216,7 +13530,7 @@
       </c>
       <c r="J197" s="6"/>
     </row>
-    <row r="198" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A198" s="6" t="s">
         <v>11</v>
       </c>
@@ -13245,7 +13559,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="199" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A199" s="13" t="s">
         <v>11</v>
       </c>
@@ -13269,7 +13583,7 @@
       </c>
       <c r="J199" s="6"/>
     </row>
-    <row r="200" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A200" s="13" t="s">
         <v>11</v>
       </c>
@@ -13293,7 +13607,7 @@
       </c>
       <c r="J200" s="6"/>
     </row>
-    <row r="201" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>11</v>
       </c>
@@ -13323,7 +13637,7 @@
       </c>
       <c r="J201" s="6"/>
     </row>
-    <row r="202" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>11</v>
       </c>
@@ -13352,7 +13666,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="203" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A203" s="6" t="s">
         <v>11</v>
       </c>
@@ -13560,7 +13874,7 @@
       </c>
       <c r="J209" s="6"/>
     </row>
-    <row r="210" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A210" s="6" t="s">
         <v>11</v>
       </c>
@@ -13590,7 +13904,7 @@
       </c>
       <c r="J210" s="6"/>
     </row>
-    <row r="211" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A211" s="6" t="s">
         <v>11</v>
       </c>
@@ -13620,7 +13934,7 @@
       </c>
       <c r="J211" s="6"/>
     </row>
-    <row r="212" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A212" s="6" t="s">
         <v>11</v>
       </c>
@@ -13650,7 +13964,7 @@
       </c>
       <c r="J212" s="6"/>
     </row>
-    <row r="213" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A213" s="6" t="s">
         <v>11</v>
       </c>
@@ -13680,7 +13994,7 @@
       </c>
       <c r="J213" s="6"/>
     </row>
-    <row r="214" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A214" s="6" t="s">
         <v>11</v>
       </c>
@@ -13710,7 +14024,7 @@
       </c>
       <c r="J214" s="6"/>
     </row>
-    <row r="215" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A215" s="6" t="s">
         <v>11</v>
       </c>
@@ -13740,7 +14054,7 @@
       </c>
       <c r="J215" s="6"/>
     </row>
-    <row r="216" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A216" s="6" t="s">
         <v>11</v>
       </c>
@@ -13830,7 +14144,7 @@
       </c>
       <c r="J218" s="6"/>
     </row>
-    <row r="219" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>11</v>
       </c>
@@ -13860,7 +14174,7 @@
       </c>
       <c r="J219" s="6"/>
     </row>
-    <row r="220" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A220" s="6" t="s">
         <v>11</v>
       </c>
@@ -13890,7 +14204,7 @@
       </c>
       <c r="J220" s="6"/>
     </row>
-    <row r="221" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>4</v>
       </c>
@@ -13920,7 +14234,7 @@
       </c>
       <c r="J221" s="6"/>
     </row>
-    <row r="222" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>4</v>
       </c>
@@ -13950,7 +14264,7 @@
       </c>
       <c r="J222" s="6"/>
     </row>
-    <row r="223" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A223" s="6" t="s">
         <v>11</v>
       </c>
@@ -13980,7 +14294,7 @@
       </c>
       <c r="J223" s="6"/>
     </row>
-    <row r="224" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A224" s="6" t="s">
         <v>11</v>
       </c>
@@ -14010,7 +14324,7 @@
       </c>
       <c r="J224" s="6"/>
     </row>
-    <row r="225" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>11</v>
       </c>
@@ -14040,7 +14354,7 @@
       </c>
       <c r="J225" s="6"/>
     </row>
-    <row r="226" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A226" s="6" t="s">
         <v>11</v>
       </c>
@@ -14070,7 +14384,7 @@
       </c>
       <c r="J226" s="6"/>
     </row>
-    <row r="227" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A227" s="6" t="s">
         <v>11</v>
       </c>
@@ -14130,7 +14444,7 @@
       </c>
       <c r="J228" s="6"/>
     </row>
-    <row r="229" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>11</v>
       </c>
@@ -14159,7 +14473,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="230" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A230" s="6" t="s">
         <v>11</v>
       </c>
@@ -14189,7 +14503,7 @@
       </c>
       <c r="J230" s="6"/>
     </row>
-    <row r="231" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A231" s="6" t="s">
         <v>11</v>
       </c>
@@ -14218,7 +14532,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="232" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>4</v>
       </c>
@@ -14248,7 +14562,7 @@
       </c>
       <c r="J232" s="6"/>
     </row>
-    <row r="233" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A233" s="6" t="s">
         <v>11</v>
       </c>
@@ -14278,7 +14592,7 @@
       </c>
       <c r="J233" s="6"/>
     </row>
-    <row r="234" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>11</v>
       </c>
@@ -14308,7 +14622,7 @@
       </c>
       <c r="J234" s="6"/>
     </row>
-    <row r="235" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>11</v>
       </c>
@@ -14430,7 +14744,7 @@
       </c>
       <c r="J238" s="6"/>
     </row>
-    <row r="239" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>11</v>
       </c>
@@ -14460,7 +14774,7 @@
       </c>
       <c r="J239" s="6"/>
     </row>
-    <row r="240" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A240" s="6" t="s">
         <v>11</v>
       </c>
@@ -14490,7 +14804,7 @@
       </c>
       <c r="J240" s="6"/>
     </row>
-    <row r="241" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A241" s="6" t="s">
         <v>11</v>
       </c>
@@ -14520,7 +14834,7 @@
       </c>
       <c r="J241" s="6"/>
     </row>
-    <row r="242" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A242" s="6" t="s">
         <v>11</v>
       </c>
@@ -14580,7 +14894,7 @@
       </c>
       <c r="J243" s="6"/>
     </row>
-    <row r="244" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>11</v>
       </c>
@@ -14610,7 +14924,7 @@
       </c>
       <c r="J244" s="6"/>
     </row>
-    <row r="245" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A245" s="6" t="s">
         <v>11</v>
       </c>
@@ -14639,7 +14953,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="246" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A246" s="6" t="s">
         <v>11</v>
       </c>
@@ -14817,7 +15131,7 @@
       </c>
       <c r="J251" s="6"/>
     </row>
-    <row r="252" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A252" s="6" t="s">
         <v>11</v>
       </c>
@@ -14847,7 +15161,7 @@
       </c>
       <c r="J252" s="6"/>
     </row>
-    <row r="253" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A253" s="6" t="s">
         <v>11</v>
       </c>
@@ -14877,7 +15191,7 @@
       </c>
       <c r="J253" s="6"/>
     </row>
-    <row r="254" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>11</v>
       </c>
@@ -14906,7 +15220,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="255" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>11</v>
       </c>
@@ -14936,7 +15250,7 @@
       </c>
       <c r="J255" s="6"/>
     </row>
-    <row r="256" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>11</v>
       </c>
@@ -14965,7 +15279,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="257" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
         <v>11</v>
       </c>
@@ -14994,7 +15308,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="258" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>11</v>
       </c>
@@ -15082,7 +15396,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="261" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A261" s="6" t="s">
         <v>11</v>
       </c>
@@ -15112,7 +15426,7 @@
       </c>
       <c r="J261" s="6"/>
     </row>
-    <row r="262" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>11</v>
       </c>
@@ -15142,7 +15456,7 @@
       </c>
       <c r="J262" s="6"/>
     </row>
-    <row r="263" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A263" s="6" t="s">
         <v>11</v>
       </c>
@@ -15172,7 +15486,7 @@
       </c>
       <c r="J263" s="6"/>
     </row>
-    <row r="264" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>11</v>
       </c>
@@ -15202,7 +15516,7 @@
       </c>
       <c r="J264" s="6"/>
     </row>
-    <row r="265" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>11</v>
       </c>
@@ -15231,7 +15545,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="266" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>11</v>
       </c>
@@ -15260,7 +15574,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="267" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>11</v>
       </c>
@@ -15290,7 +15604,7 @@
       </c>
       <c r="J267" s="6"/>
     </row>
-    <row r="268" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A268" s="2" t="s">
         <v>11</v>
       </c>
@@ -15380,7 +15694,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="271" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A271" s="6" t="s">
         <v>11</v>
       </c>
@@ -15410,7 +15724,7 @@
       </c>
       <c r="J271" s="6"/>
     </row>
-    <row r="272" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A272" s="6" t="s">
         <v>11</v>
       </c>
@@ -15440,7 +15754,7 @@
       </c>
       <c r="J272" s="6"/>
     </row>
-    <row r="273" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A273" s="2" t="s">
         <v>11</v>
       </c>
@@ -15469,7 +15783,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="274" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A274" s="2" t="s">
         <v>11</v>
       </c>
@@ -15559,7 +15873,7 @@
       </c>
       <c r="J276" s="6"/>
     </row>
-    <row r="277" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>11</v>
       </c>
@@ -15589,7 +15903,7 @@
       </c>
       <c r="J277" s="6"/>
     </row>
-    <row r="278" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
         <v>11</v>
       </c>
@@ -15618,7 +15932,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="279" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>11</v>
       </c>
@@ -15648,7 +15962,7 @@
       </c>
       <c r="J279" s="2"/>
     </row>
-    <row r="280" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A280" s="6" t="s">
         <v>11</v>
       </c>
@@ -15680,7 +15994,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="281" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A281" s="6" t="s">
         <v>11</v>
       </c>
@@ -15712,7 +16026,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="282" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A282" s="6" t="s">
         <v>11</v>
       </c>
@@ -15953,7 +16267,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="290" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A290" s="6" t="s">
         <v>11</v>
       </c>
@@ -15982,7 +16296,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="291" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A291" s="6" t="s">
         <v>11</v>
       </c>
@@ -16011,7 +16325,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="292" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A292" s="6" t="s">
         <v>11</v>
       </c>
@@ -16041,7 +16355,7 @@
       </c>
       <c r="J292" s="6"/>
     </row>
-    <row r="293" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
         <v>11</v>
       </c>
@@ -16071,7 +16385,7 @@
       </c>
       <c r="J293" s="6"/>
     </row>
-    <row r="294" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A294" s="6" t="s">
         <v>11</v>
       </c>
@@ -16101,7 +16415,7 @@
       </c>
       <c r="J294" s="6"/>
     </row>
-    <row r="295" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A295" s="6" t="s">
         <v>11</v>
       </c>
@@ -16130,7 +16444,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="296" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A296" s="6" t="s">
         <v>11</v>
       </c>
@@ -16159,7 +16473,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="297" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A297" s="6" t="s">
         <v>11</v>
       </c>
@@ -16212,7 +16526,7 @@
       </c>
       <c r="J298" s="6"/>
     </row>
-    <row r="299" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A299" s="6" t="s">
         <v>11</v>
       </c>
@@ -16240,7 +16554,7 @@
       </c>
       <c r="J299" s="6"/>
     </row>
-    <row r="300" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A300" s="6" t="s">
         <v>11</v>
       </c>
@@ -16264,7 +16578,7 @@
         <v>3250</v>
       </c>
     </row>
-    <row r="301" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
         <v>4</v>
       </c>
@@ -16293,7 +16607,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="302" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A302" s="6" t="s">
         <v>4</v>
       </c>
@@ -16322,7 +16636,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="303" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
         <v>4</v>
       </c>
@@ -16352,7 +16666,7 @@
       </c>
       <c r="J303" s="6"/>
     </row>
-    <row r="304" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A304" s="6" t="s">
         <v>11</v>
       </c>
@@ -16382,7 +16696,7 @@
       </c>
       <c r="J304" s="6"/>
     </row>
-    <row r="305" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A305" s="6" t="s">
         <v>11</v>
       </c>
@@ -16411,7 +16725,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="306" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
         <v>4</v>
       </c>
@@ -16443,7 +16757,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="307" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>4</v>
       </c>
@@ -16473,7 +16787,7 @@
       </c>
       <c r="J307" s="6"/>
     </row>
-    <row r="308" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
         <v>4</v>
       </c>
@@ -16502,7 +16816,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="309" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
         <v>4</v>
       </c>
@@ -16531,7 +16845,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="310" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
         <v>4</v>
       </c>
@@ -16560,7 +16874,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="311" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
         <v>4</v>
       </c>
@@ -16590,7 +16904,7 @@
       </c>
       <c r="J311" s="6"/>
     </row>
-    <row r="312" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A312" s="6" t="s">
         <v>11</v>
       </c>
@@ -16619,7 +16933,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="313" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A313" s="6" t="s">
         <v>4</v>
       </c>
@@ -16649,7 +16963,7 @@
       </c>
       <c r="J313" s="6"/>
     </row>
-    <row r="314" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A314" s="6" t="s">
         <v>11</v>
       </c>
@@ -16679,7 +16993,7 @@
       </c>
       <c r="J314" s="6"/>
     </row>
-    <row r="315" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A315" s="6" t="s">
         <v>11</v>
       </c>
@@ -16708,7 +17022,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="316" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
         <v>4</v>
       </c>
@@ -16738,7 +17052,7 @@
       </c>
       <c r="J316" s="6"/>
     </row>
-    <row r="317" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A317" s="6" t="s">
         <v>11</v>
       </c>
@@ -16768,7 +17082,7 @@
       </c>
       <c r="J317" s="6"/>
     </row>
-    <row r="318" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A318" s="6" t="s">
         <v>11</v>
       </c>
@@ -16797,7 +17111,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="319" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A319" s="6" t="s">
         <v>11</v>
       </c>
@@ -16827,7 +17141,7 @@
       </c>
       <c r="J319" s="6"/>
     </row>
-    <row r="320" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
         <v>4</v>
       </c>
@@ -16857,7 +17171,7 @@
       </c>
       <c r="J320" s="6"/>
     </row>
-    <row r="321" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
         <v>4</v>
       </c>
@@ -16886,7 +17200,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="322" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A322" t="s">
         <v>4</v>
       </c>
@@ -16916,7 +17230,7 @@
       </c>
       <c r="J322" s="6"/>
     </row>
-    <row r="323" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A323" t="s">
         <v>4</v>
       </c>
@@ -16946,7 +17260,7 @@
       </c>
       <c r="J323" s="6"/>
     </row>
-    <row r="324" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A324" t="s">
         <v>4</v>
       </c>
@@ -16975,7 +17289,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="325" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A325" t="s">
         <v>4</v>
       </c>
@@ -17005,7 +17319,7 @@
       </c>
       <c r="J325" s="6"/>
     </row>
-    <row r="326" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A326" s="6" t="s">
         <v>11</v>
       </c>
@@ -17035,7 +17349,7 @@
       </c>
       <c r="J326" s="6"/>
     </row>
-    <row r="327" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A327" s="6" t="s">
         <v>11</v>
       </c>
@@ -17065,7 +17379,7 @@
       </c>
       <c r="J327" s="6"/>
     </row>
-    <row r="328" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A328" s="6" t="s">
         <v>11</v>
       </c>
@@ -17095,7 +17409,7 @@
       </c>
       <c r="J328" s="6"/>
     </row>
-    <row r="329" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A329" s="6" t="s">
         <v>11</v>
       </c>
@@ -17125,7 +17439,7 @@
       </c>
       <c r="J329" s="6"/>
     </row>
-    <row r="330" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A330" s="6" t="s">
         <v>11</v>
       </c>
@@ -17155,7 +17469,7 @@
       </c>
       <c r="J330" s="6"/>
     </row>
-    <row r="331" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A331" s="6" t="s">
         <v>11</v>
       </c>
@@ -17184,7 +17498,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="332" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A332" s="6" t="s">
         <v>11</v>
       </c>
@@ -17214,7 +17528,7 @@
       </c>
       <c r="J332" s="6"/>
     </row>
-    <row r="333" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A333" s="6" t="s">
         <v>11</v>
       </c>
@@ -17243,7 +17557,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="334" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A334" s="13" t="s">
         <v>11</v>
       </c>
@@ -17273,7 +17587,7 @@
       </c>
       <c r="J334" s="6"/>
     </row>
-    <row r="335" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A335" t="s">
         <v>4</v>
       </c>
@@ -17303,7 +17617,7 @@
       </c>
       <c r="J335" s="6"/>
     </row>
-    <row r="336" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A336" t="s">
         <v>4</v>
       </c>
@@ -17332,7 +17646,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="337" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A337" t="s">
         <v>4</v>
       </c>
@@ -17362,7 +17676,7 @@
       </c>
       <c r="J337" s="6"/>
     </row>
-    <row r="338" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A338" t="s">
         <v>4</v>
       </c>
@@ -17391,7 +17705,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="339" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A339" t="s">
         <v>4</v>
       </c>
@@ -17421,7 +17735,7 @@
       </c>
       <c r="J339" s="6"/>
     </row>
-    <row r="340" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A340" t="s">
         <v>4</v>
       </c>
@@ -17450,7 +17764,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="341" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A341" t="s">
         <v>4</v>
       </c>
@@ -17479,7 +17793,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="342" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A342" s="6" t="s">
         <v>11</v>
       </c>
@@ -17509,7 +17823,7 @@
       </c>
       <c r="J342" s="6"/>
     </row>
-    <row r="343" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A343" s="6" t="s">
         <v>11</v>
       </c>
@@ -17538,7 +17852,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="344" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A344" s="6" t="s">
         <v>11</v>
       </c>
@@ -17567,7 +17881,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="345" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A345" s="13" t="s">
         <v>11</v>
       </c>
@@ -17591,7 +17905,7 @@
       </c>
       <c r="J345" s="6"/>
     </row>
-    <row r="346" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A346" t="s">
         <v>4</v>
       </c>
@@ -17621,7 +17935,7 @@
       </c>
       <c r="J346" s="6"/>
     </row>
-    <row r="347" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A347" s="6" t="s">
         <v>11</v>
       </c>
@@ -17651,7 +17965,7 @@
       </c>
       <c r="J347" s="6"/>
     </row>
-    <row r="348" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A348" t="s">
         <v>4</v>
       </c>
@@ -17681,7 +17995,7 @@
       </c>
       <c r="J348" s="6"/>
     </row>
-    <row r="349" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A349" t="s">
         <v>4</v>
       </c>
@@ -17711,7 +18025,7 @@
       </c>
       <c r="J349" s="6"/>
     </row>
-    <row r="350" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A350" t="s">
         <v>4</v>
       </c>
@@ -17741,7 +18055,7 @@
       </c>
       <c r="J350" s="6"/>
     </row>
-    <row r="351" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A351" t="s">
         <v>4</v>
       </c>
@@ -17771,7 +18085,7 @@
       </c>
       <c r="J351" s="6"/>
     </row>
-    <row r="352" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A352" s="6" t="s">
         <v>11</v>
       </c>
@@ -17801,7 +18115,7 @@
       </c>
       <c r="J352" s="6"/>
     </row>
-    <row r="353" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A353" s="6" t="s">
         <v>11</v>
       </c>
@@ -17831,7 +18145,7 @@
       </c>
       <c r="J353" s="6"/>
     </row>
-    <row r="354" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A354" s="13" t="s">
         <v>130</v>
       </c>
@@ -17861,7 +18175,7 @@
       </c>
       <c r="J354" s="6"/>
     </row>
-    <row r="355" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A355" s="13" t="s">
         <v>130</v>
       </c>
@@ -17891,7 +18205,7 @@
       </c>
       <c r="J355" s="6"/>
     </row>
-    <row r="356" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A356" s="13" t="s">
         <v>130</v>
       </c>
@@ -17921,7 +18235,7 @@
       </c>
       <c r="J356" s="6"/>
     </row>
-    <row r="357" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A357" s="13" t="s">
         <v>130</v>
       </c>
@@ -17951,7 +18265,7 @@
       </c>
       <c r="J357" s="6"/>
     </row>
-    <row r="358" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A358" s="13" t="s">
         <v>130</v>
       </c>
@@ -17981,7 +18295,7 @@
       </c>
       <c r="J358" s="6"/>
     </row>
-    <row r="359" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A359" s="13" t="s">
         <v>130</v>
       </c>
@@ -18011,7 +18325,7 @@
       </c>
       <c r="J359" s="6"/>
     </row>
-    <row r="360" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A360" s="13" t="s">
         <v>130</v>
       </c>
@@ -18040,7 +18354,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="361" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A361" s="13" t="s">
         <v>130</v>
       </c>
@@ -18069,7 +18383,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="362" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A362" s="13" t="s">
         <v>130</v>
       </c>
@@ -18099,7 +18413,7 @@
       </c>
       <c r="J362" s="6"/>
     </row>
-    <row r="363" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A363" s="13" t="s">
         <v>130</v>
       </c>
@@ -18128,7 +18442,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="364" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A364" s="13" t="s">
         <v>130</v>
       </c>
@@ -18158,7 +18472,7 @@
       </c>
       <c r="J364" s="6"/>
     </row>
-    <row r="365" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A365" s="13" t="s">
         <v>130</v>
       </c>
@@ -18187,7 +18501,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="366" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A366" s="13" t="s">
         <v>130</v>
       </c>
@@ -18216,7 +18530,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="367" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A367" s="13" t="s">
         <v>130</v>
       </c>
@@ -18245,7 +18559,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="368" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A368" s="13" t="s">
         <v>130</v>
       </c>
@@ -18275,7 +18589,7 @@
       </c>
       <c r="J368" s="6"/>
     </row>
-    <row r="369" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A369" s="13" t="s">
         <v>130</v>
       </c>
@@ -18305,7 +18619,7 @@
       </c>
       <c r="J369" s="6"/>
     </row>
-    <row r="370" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A370" s="13" t="s">
         <v>130</v>
       </c>
@@ -18335,7 +18649,7 @@
       </c>
       <c r="J370" s="6"/>
     </row>
-    <row r="371" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A371" s="13" t="s">
         <v>130</v>
       </c>
@@ -18364,7 +18678,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="372" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A372" s="13" t="s">
         <v>130</v>
       </c>
@@ -18394,7 +18708,7 @@
       </c>
       <c r="J372" s="6"/>
     </row>
-    <row r="373" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A373" s="13" t="s">
         <v>130</v>
       </c>
@@ -18424,7 +18738,7 @@
       </c>
       <c r="J373" s="6"/>
     </row>
-    <row r="374" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A374" s="13" t="s">
         <v>130</v>
       </c>
@@ -18454,7 +18768,7 @@
       </c>
       <c r="J374" s="6"/>
     </row>
-    <row r="375" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A375" s="13" t="s">
         <v>130</v>
       </c>
@@ -18484,7 +18798,7 @@
       </c>
       <c r="J375" s="6"/>
     </row>
-    <row r="376" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A376" s="13" t="s">
         <v>130</v>
       </c>
@@ -18514,7 +18828,7 @@
       </c>
       <c r="J376" s="6"/>
     </row>
-    <row r="377" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A377" s="13" t="s">
         <v>130</v>
       </c>
@@ -18740,11 +19054,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I377" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="LMB"/>
-      </filters>
-    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A53:I298">
       <sortCondition ref="G1:G377"/>
     </sortState>
@@ -24750,6 +25059,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010008813DEC4A17DB40A5843D1157D8CD4D" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dc6577e42519716f75255cf7493b32f7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9" xmlns:ns3="7ce4cce1-0673-44d6-a8e9-024984c6c156" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="93d8227084f1dc13f4d26d22ce1da744" ns2:_="" ns3:_="">
     <xsd:import namespace="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9"/>
@@ -25004,15 +25322,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -25025,6 +25334,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0785BFC6-745B-49B0-87B9-892A72BBB88F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3258F12-C15B-4654-A491-0335704C572D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -25039,14 +25356,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0785BFC6-745B-49B0-87B9-892A72BBB88F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
v1.24 Added table script
Added a separate script that produces a summary and results table, and removed code from plotting script that originally did this.
</commit_message>
<xml_diff>
--- a/01_data/01_raw_files/Fixed_fish_widths_DraftExcelAnalysis_Feb2026.xlsx
+++ b/01_data/01_raw_files/Fixed_fish_widths_DraftExcelAnalysis_Feb2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RIZZUTOM\Desktop\GitHub Projects\2026_Reddick_fish_morphology\01_data\01_raw_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05ADED76-59D3-4CC3-9A91-89F50073B927}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{843C6589-ECDE-4793-94A5-C58083C25822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7878,7 +7878,7 @@
         <v>45958</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="F17" s="6">
         <v>241</v>
@@ -8063,31 +8063,31 @@
       </c>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="A23" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B23" s="6" t="s">
+      <c r="A23" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B23" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="C23" t="s">
-        <v>125</v>
-      </c>
-      <c r="D23" s="10">
+      <c r="C23" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="D23" s="14">
         <v>45945</v>
       </c>
-      <c r="E23" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="F23" s="6">
+      <c r="E23" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F23" s="13">
         <v>200</v>
       </c>
-      <c r="G23" s="6">
+      <c r="G23" s="13">
         <v>32</v>
       </c>
-      <c r="H23" s="6">
+      <c r="H23" s="13">
         <v>250</v>
       </c>
-      <c r="I23" s="6" t="s">
+      <c r="I23" s="13" t="s">
         <v>88</v>
       </c>
       <c r="J23" s="6"/>
@@ -8109,7 +8109,7 @@
         <v>45945</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="F24" s="6">
         <v>200</v>
@@ -8129,29 +8129,29 @@
       </c>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="A25" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B25" s="6" t="s">
+      <c r="A25" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="C25" t="s">
-        <v>125</v>
-      </c>
-      <c r="D25" s="10">
+      <c r="C25" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="D25" s="14">
         <v>45945</v>
       </c>
-      <c r="E25" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="F25" s="6">
+      <c r="E25" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F25" s="13">
         <v>192</v>
       </c>
-      <c r="G25" s="6">
+      <c r="G25" s="13">
         <v>21</v>
       </c>
-      <c r="H25" s="6">
-        <v>29</v>
+      <c r="H25" s="13">
+        <v>129</v>
       </c>
       <c r="I25" s="6" t="s">
         <v>88</v>
@@ -8172,7 +8172,7 @@
         <v>45945</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="F26" s="6">
         <v>180</v>
@@ -10903,7 +10903,7 @@
         <v>45944</v>
       </c>
       <c r="E109" s="6" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="F109" s="6">
         <v>241</v>
@@ -15440,7 +15440,7 @@
         <v>45791</v>
       </c>
       <c r="E262" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="F262">
         <v>104</v>
@@ -25059,15 +25059,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010008813DEC4A17DB40A5843D1157D8CD4D" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dc6577e42519716f75255cf7493b32f7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9" xmlns:ns3="7ce4cce1-0673-44d6-a8e9-024984c6c156" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="93d8227084f1dc13f4d26d22ce1da744" ns2:_="" ns3:_="">
     <xsd:import namespace="cb7bf1ad-b1cc-435a-9f6e-81b2f99c32a9"/>
@@ -25322,6 +25313,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -25334,14 +25334,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0785BFC6-745B-49B0-87B9-892A72BBB88F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3258F12-C15B-4654-A491-0335704C572D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -25356,6 +25348,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0785BFC6-745B-49B0-87B9-892A72BBB88F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>